<commit_message>
Add FLOOD-011 to FLOOD-020 to Flood Case Database - Batch 2 complete
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Flood_Case_Database.xlsx
+++ b/knowledge/case-databases/Flood_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1653,6 +1653,1056 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="120" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>DRN2341674</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>5 Jul 2017</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Static caravan destroyed by flooding at caravan park following major storm; flood exclusion endorsement applied at inception; claimant argued storm was proximate cause</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>River burst banks due to cumulative heavy rainfall over 2 months prior to storm; storm occurred on already-saturated ground; ground-level floodwater from river inundated caravan park</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Other (static caravan / holiday park)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Specific flood exclusion endorsement applied at inception due to high flood risk at caravan park; flood was proximate cause of damage, not storm — cumulative rainfall caused river to rise, storm was not the active and efficient cause</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Claimant argued storm was proximate cause and but-for storm flood would not have occurred; insurer cited 2 months of heavy rainfall saturating ground and Met Office data; damage caused solely by floodwater not by storm action</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — flood exclusion endorsement at inception valid and clearly communicated; proximate cause of damage was flood (cumulative rainfall), not storm as a single event; insurer not required to cover claim</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>Flood exclusion endorsement specific to caravan park (high-risk location); proximate cause test — heavy rainfall over preceding months was the active and efficient cause of the river flooding, not the storm; 'but for' test insufficient where independent cause (cumulative rainfall) would likely have produced same result</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>No independent hydrological report distinguishing storm contribution from pre-existing rainfall accumulation; no evidence storm alone would have caused flood absent prior saturation</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>Heavy rainfall 2 months before storm saturated ground; river likely to have burst regardless of storm; damage caused solely by floodwater — if barriers had been in place, storm alone would not have caused damage; claimant agreed to flood endorsement terms at inception; 'but for' storm argument fails because prior rainfall was itself an independent operative cause</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>Specific flood endorsements at inception are enforceable even when storm immediately precedes flood; proximate cause test requires identifying the efficient cause of the flood itself (not just the triggering weather event); cumulative prior rainfall qualifying as an independent cause defeats the 'but for storm' argument</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>IF flood_exclusion_endorsed_at_inception = TRUE AND proximate_cause = 'flood' AND cumulative_prior_rainfall_was_independent_cause THEN decline; storm as contributing factor insufficient to override explicit endorsement</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>DRN2341674.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="120" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-012</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>DRN2449131</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Woodland Insurance Services Ltd</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>11 Dec 2015</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Broker conduct dispute — broker failed to properly disclose prior flood history to insurer causing insurer to remove flood cover and decline commercial property flood claim (2014 heavy rain, drain overflow)</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Surface water / drain overflow — drains unable to cope with heavy rainfall; water entered ground floor of commercial buy-to-let property; culvert blocked causing water to overflow and enter premises</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Commercial (buy-to-let rental)</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Insurer removed flood cover and declined claim after discovering undisclosed flood history (two prior floods in 2007 and 2012); broker had described prior events as 'blocked drains' rather than flooding, understating the risk</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Broker claimed Mr R only mentioned 'blocked drains'; Mr R said he disclosed full flood history and showed conveyancer documents; call recording confirmed broker knew dates and water company involvement — sufficient to trigger duty to investigate further; broker's own post-decline letter referenced culvert flooding inconsistent with 'only just learned' defence</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>Complaint upheld against broker — broker should have disclosed or further investigated flood history before submitting to insurer; insurer separately directed to consider claim; broker to pay Mr R £100 for trouble and upset caused by delay</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="inlineStr">
+        <is>
+          <t>Broker's duty to accurately communicate material prior flood history to insurer; duty to probe ambiguous prior claim descriptions; client entitled to rely on broker's competence in handling disclosure</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="inlineStr">
+        <is>
+          <t>No written record of what Mr R disclosed during face-to-face broker visit; call recording available but confirmed 'blocked drains' framing despite broker knowing dates and water company context</t>
+        </is>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
+        <is>
+          <t>Broker knew the dates and water company's remedial works — this information came from Mr R and was sufficient to trigger further enquiry; 'blocked drains' framing understated risk; Mr R had no incentive to downplay severity; broker's post-decline letter referencing culvert flooding undermined defence that full facts were not known at outset; Mr R entitled to assume questions were answered correctly having signed summary on broker's advice</t>
+        </is>
+      </c>
+      <c r="S13" s="5" t="inlineStr">
+        <is>
+          <t>Brokers must probe ambiguous prior claim descriptions; 'blocked drains' terminology can conceal material flood history — any description involving internal water damage or prior claims should prompt specific flood disclosure questions; signing a statement of fact prepared by the broker does not shift responsibility to the client</t>
+        </is>
+      </c>
+      <c r="T13" s="5" t="inlineStr">
+        <is>
+          <t>IF prior_claim_described_as_blocked_drains AND internal_flooding_known_or_inferable THEN broker_must_verify_flood_classification_before_submission_to_insurer; IF broker_has_dates_and_remediation_detail THEN duty_to_investigate_triggered</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>DRN2449131.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2482936</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>5 Apr 2021</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Peril classification dispute — AXA classified claim as flood after flash flood caused drain backup and internal water ingress; policyholders argued classification should be escape of water from blocked drain, fearing adverse impact on future premiums and resale value</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>External surface water / flash flood — exceptionally heavy rainfall caused drains to back up unable to cope with volume; rainwater unable to enter drain accumulated outside and entered property; no standing water observed at time of loss adjuster visit</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Peril Classification Dispute</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — claim accepted and repaired under flood peril; policyholders disputed classification only (concerned about premium and resale impact)</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Policyholders argued drain was blocked by building debris before rain (escape of water); AXA cited flash flood evidence including regional claims data and very heavy rainfall in preceding days; policyholders provided river level data showing levels had previously been higher without water ingress; no emergency plumber's report retained</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — AXA's flood classification upheld; proximate cause was external rainwater flooding the ground outside; water never entered the drain so cannot be escape of water; river level data irrelevant to local circumstances; absence of plumber's report immaterial</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>Flood defined as 'invasion of property by large volume of water caused by rapid build-up or sudden release of water from outside the buildings'; escape of water requires water to have entered and then escaped an apparatus — water that never entered the drain cannot escape from it; proximate cause is the external rainwater flooding the ground, not a blockage within the drainage apparatus</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>Emergency plumber's report not retained by AXA (AXA arranged the plumber); CCTV drain survey to confirm pre-existing blockage vs. flood-induced backup; plumber's report would not have changed outcome given undisputed that water could not enter drain</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>Flash flood confirmed by regional claims data and heavy rainfall evidence; drain backed up because it could not cope with rainfall volume — flood overwhelmed drainage; water that cannot enter the drain has not 'escaped' from it; escape of water requires release from apparatus containing water, not failure of drainage to absorb external water; local river level data does not determine whether local circumstances constituted a flood; AXA acted reasonably in its classification</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>Flood vs EOW classification turns on whether water entered the drain/pipe (EOW) or was unable to enter at all (flood); absence of plumber's report does not change outcome where cause is undisputed; consumer concern about premium and resale impact does not alter correct peril classification</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>IF external_surface_water_confirmed = TRUE AND water_unable_to_enter_drain = TRUE THEN classify_as_flood NOT escape_of_water; escape_of_water requires prior containment within apparatus</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2482936.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="120" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-014</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>DRN2512341</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Zurich Insurance PLC</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>28 Feb 2019</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Latent flood damage claim — wet rot on joists discovered after purchase; previous owner had a 'serious flood' approximately 2 years before; claimant sought to invoke secondary flooding protocol; Zurich declined as damage pre-dated policy inception</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Unknown — original cause unconfirmed; possibly escape of water (pipe/appliance) or external flood; property not near river; no evidence of damage to neighbouring properties consistent with natural flood</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Pre-Inception Damage Dispute</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Damage occurred before policy inception; secondary flooding protocol requires confirmed flood as original cause — cannot establish on balance of probabilities that original damage was caused by flood rather than escape of water; escape of water is the more likely cause given property location; secondary escape of water not covered by secondary flooding protocol</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Only hearsay from neighbour that previous owner had 'serious flood'; no access to original claim file; property not near river or body of water; no evidence of damage to neighbouring properties; claimant later noted property in medium-high surface water flood risk area and found water in floor void during renovation — FOS found this did not add to case</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Zurich's decline upheld; secondary flooding protocol does not apply where original cause unconfirmed; escape of water more likely given location and absence of neighbouring flood damage; hearsay from neighbour insufficient to establish balance of probabilities; water found during renovation not linked to original damage</t>
+        </is>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>Coverage limited to damage occurring during policy period; secondary flooding protocol (industry practice) applies only to confirmed flood damage — does not extend to secondary escape of water; even if escape of water causes a flood, predominant cause remains escape of water; policyholder must show on balance of probabilities that original damage was caused by flood</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Original claim file from previous owner's insurer; professional confirmation of how original damage was classified (flood or EOW); hydrological flood risk mapping for the specific property; evidence of flood damage to neighbouring properties at the relevant time</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Neighbour hearsay insufficient — 'serious flood' ambiguous as to cause, extent, and mechanism; property not near natural water body; no evidence neighbouring properties were damaged suggesting natural flood; escape of water scenario more consistent with property location; subsequent water found in floor void during renovation not conclusively linked to original damage or to flood; secondary flooding protocol narrow and confirmed-flood-only</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>To invoke secondary flooding protocol, claimant must establish on balance of probabilities that original damage was caused by flood (not merely that a flood happened); property location, absence of neighbouring damage, and classification of original claim are key factors; hearsay from a neighbour is insufficient; the distinction between flood and escape of water matters even when the practical outcome is similar</t>
+        </is>
+      </c>
+      <c r="T15" s="5" t="inlineStr">
+        <is>
+          <t>IF latent_damage_pre_policy = TRUE AND original_cause_unconfirmed THEN decline_secondary_flooding_protocol UNLESS flood_established_on_balance_of_probabilities_by_evidence_beyond_hearsay</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>DRN2512341.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="120" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2541699</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>The National Farmers' Union Mutual Insurance Society Limited</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>23 Feb 2021</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Peril classification dispute — NFUM classified water-soaked carpet as flood leading to Flood Re cession and near-doubled renewal premium; claimant argued storm was main cause as rainfall was of exceptional intensity; inadequate loss adjuster investigation</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Surface water ingress — carpet soaked in corner of sitting room after exceptionally heavy rain (15.4mm/hour); entry point not inspected by loss adjuster; possibly gutter overflow or drain backup; no standing water accumulation observed at loss adjuster visit 9 days later</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Peril Classification Dispute</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — claim accepted and carpet paid (approx £1,100); dispute is classification: NFUM classified as flood leading to Flood Re cession and large premium increase; claimant sought reclassification as storm</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Loss adjuster concluded flood (drains backed up) based on inspection 9 days post-incident with no drain or gutter inspection; weather records showed 15.4mm/hour rainfall (exceptional intensity) on the day; no evidence of standing water accumulation required for NFUM's flood definition; claimant argued storm caused damage via gutter overflow</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>Complaint upheld — storm reclassified as main cause; NFUM to reclassify claim as storm, update records including external databases, reassess and rewrite 2020/21 policy cover, refund excess premium with 8% simple interest per annum, and withdraw policy from Flood Re scheme</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>Storm (no policy definition — FOS applies: violent winds or exceptional intensity rainfall; 15.4mm/hour qualifies); NFUM flood definition requires substantial/abnormal body of water entering at ground level — no evidence of standing accumulation; Flood Re cession criteria require a flood claim; where both storm and flood could apply, FOS assesses which was main cause</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>Loss adjuster did not inspect drain or gutter at time of claim; no record of whether standing water accumulation was present at time of damage (visited 9 days later); loss adjuster report conclusory and did not explain how flood determination was reached; no gutter or drain inspection conducted</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="inlineStr">
+        <is>
+          <t>15.4mm/hour rainfall = exceptional intensity constituting a storm; NFUM's own flood definition requires substantial/abnormal body of water — no evidence of standing accumulation at time of damage; loss adjuster's report inadequate — visited 9 days post-incident with no drain or gutter inspection; given drastic premium consequences of flood classification and probability that damage was caused by storm, fair to reclassify; NFUM's underwriting technician's reliance on 'drains backed up' finding in inadequate report insufficient to maintain flood classification</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>When flood vs storm classification triggers Flood Re cession and large premium increase, FOS applies heightened scrutiny to adequacy of loss adjuster investigation; a conclusory report produced after 9-day delay without drain or gutter inspection cannot support flood classification where storm evidence (weather records) is strong; insurers must conduct contemporaneous thorough investigations before classifying perils with significant premium consequences</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>IF rainfall_intensity &gt;= 15mm_per_hour AND no_standing_water_evidenced AND loss_adjuster_inspection_inadequate_or_delayed THEN consider_storm_reclassification; IF flood_classification_triggers_flood_re_cession THEN require_adequate_contemporaneous_investigation_before_flood_classification_stands</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2541699.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-016</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2632381</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>29 Mar 2021</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Commercial basement flood claim declined — RSA applied rising water table exclusion; claimant argued heavy rain was proximate cause and exclusion should not apply</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Rising water table / groundwater — prolonged heavy rainfall raised water table to basement level; basement (recently tanked) inundated; contractor confirmed cause was 'rising groundwater associated with rainfall and water table changes'</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Commercial (rental property with basement)</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Rising water table exclusion in policy — flooding caused by change in groundwater/water table level; contractor's own evidence confirmed rising groundwater as cause; prior tanking consistent with known groundwater vulnerability; heavy rain as contributing cause does not override explicit exclusion for water table mechanism</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Claimant argued heavy rain was proximate cause and causal link between rainfall and water table rise should engage flood cover; contractor's evidence attributed flooding to rainfall and water table changes; RSA relied on exclusion wording and contractor's own description of the mechanism</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — RSA's application of rising water table exclusion upheld; causal link between heavy rain and water table rise acknowledged but does not override the explicit exclusion; contractor's evidence itself confirmed the exclusion mechanism; insurer met burden of showing exclusion applies on balance of probabilities</t>
+        </is>
+      </c>
+      <c r="N17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>Explicit exclusion for loss or damage caused by rising water table levels; onus on insurer to show exclusion applies on balance of probabilities; rising water table exclusion not unusual in commercial property policies; even if heavy rain caused the water table to rise, the mechanism of water entry (rising groundwater) falls within the exclusion</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>No independent hydrological report distinguishing groundwater flood from surface water flood; contractor's report was the only professional evidence — and it supported the exclusion mechanism; no evidence of surface water entry independent of the water table rise</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>Contractor explicitly described cause as rising groundwater associated with rainfall — this is the exclusion mechanism; tanking already installed indicates known groundwater vulnerability; while heavy rain contributed, this does not change the mechanism of entry; RSA's exclusion is clear and not unusual for commercial policies; insurer met burden on balance of probabilities via contractor's own evidence; causal link between rain and water table rise is direct but does not negate the exclusion</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>Rising water table exclusion is enforceable even where heavy rain ultimately caused the water table to rise; policyholders with basements in groundwater-susceptible areas should be alerted to this exclusion at point of sale or renewal; prior installation of tanking is consistent with known groundwater risk and supports application of exclusion</t>
+        </is>
+      </c>
+      <c r="T17" s="5" t="inlineStr">
+        <is>
+          <t>IF flood_mechanism = 'groundwater_rise' AND rising_water_table_exclusion_in_policy = TRUE THEN decline EVEN IF prolonged_rainfall_was_contributing_cause; onus_on_insurer_to_show_exclusion_applies_on_balance_of_probabilities</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2632381.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="120" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2785967</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Ageas Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>9 Jul 2021</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Flood claim declined — Ageas argued damage was limited to garden/riverbank (uncovered) after August 2020 flood caused riverbank erosion; claimant contended a garden wall (covered building element) was destroyed</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>River flooding / bank erosion — property at confluence of two rivers; heavy rain in August 2020 caused riverbank at end of garden to collapse into river; county council drainage engineer confirmed flooding event; structural engineer confirmed flood causation</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Damage limited to garden/riverbank — not covered under buildings definition; insufficient evidence that a garden wall (a covered building element per policy definition) was present and destroyed by the flood; policyholder bears burden of showing covered property was damaged</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Claimant asserted permanent stone garden wall on stone foundations existed at riverbank (partially vegetation-covered; lower sections/foundations not visible); none of initial expert reports (council engineer, structural engineer, loss adjuster) mentioned a wall; repair engineer later referenced 'remains of existing damaged block stone foundation and stone wall'; insurance risk manager used uncertain language ('able to ascertain remains of a stone wall'); initial call to Ageas described riverbank collapse not wall; daughter mentioned gabions and boulders but not a wall</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — burden of proof not met; insufficient evidence that a covered building structure (garden wall) was damaged by flood as opposed to uncovered garden/riverbank; no contemporaneous expert confirmed wall existed; policyholder must show on balance that covered property was damaged by insured event; no award</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>Policy buildings definition includes garden walls but not garden items (flower beds, hedges, lawns, shrubs, trees); burden on policyholder to show on balance of probabilities that a covered property element was damaged by an insured event; Ageas not required to prove absence of a wall — policyholder must prove presence of covered structure</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>Pre-flood photographs or structural survey confirming existence and classification of a garden wall; contemporaneous inspection report from council or structural engineer mentioning wall; CCTV or survey of riverbank prior to flood; no expert who attended the site before or immediately after the flood mentioned a wall</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>No contemporaneous expert confirmed a garden wall; multiple early expert reports (council engineer, structural engineer, loss adjuster) silent on any wall despite detailed inspections; Mr J's own initial report to Ageas described riverbank collapse only; daughter mentioned gabions and boulders; insurance risk manager's language implied uncertainty; repair engineer only saw damaged remains post-flood making pre-flood description unreliable; structure only partially visible (vegetation-covered) before flood creating unrecoverable evidential gap</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>Claims for flood damage to garden structures require pre-loss documentary evidence of the structure's existence and its eligibility as a covered building element; structures partially obscured by vegetation or only partially visible present an unrecoverable evidential gap if not pre-documented; multiple contemporaneous expert visits without mention of a wall is strong evidence against its existence as a covered structure</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>IF claimed_damaged_structure_not_mentioned_in_contemporaneous_expert_reports AND no_pre_loss_documentation_of_covered_structure THEN burden_of_proof_not_met AND decline; policyholder_must_prove_covered_property_was_damaged_on_balance_of_probabilities</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2785967.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="120" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-018</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2787998</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Ocaso SA, Compania de Seguros y Reaseguros</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>11 Jun 2021</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Flood claim declined — Ocaso retrospectively excluded flood cover after Ms J disclosed 1998 area flood history; flood exclusion endorsement added December 2019; property flooded February 2020 following named storm</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>External flooding following named storm (February 2020); property confirmed high flood risk by government data; area had flooded in 1998 when nearby river burst its banks</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Flood cover excluded by endorsement added December 2019 (retrospective to inception August 2018) after Ms J disclosed 1998 flood history; insurer's underwriting guidelines demonstrate it would never have offered flood cover if prior flood history had been known; property confirmed as high flood risk by government website; answers at inception were inaccurate even if given in good faith</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Ms J argued she was unaware of 1998 flood history when taking out policy (lived there after); answered flood risk questions to best of knowledge at time; Ocaso provided underwriting guidelines confirming it would never have offered flood cover for this risk; government website confirmed property at high flood risk; Ms J argued neighbour with Ocaso policy was covered for flood</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — flood exclusion endorsement fairly applied retrospectively; inaccurate answers at inception (even in good faith) are material; Ocaso demonstrated via underwriting guidelines it would not have offered flood cover; broker instructed to notify Ms J of change; claim fairly declined; Flood Re not available via price comparison site route; neighbour's policy circumstances not comparable</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>Material change in risk — prior flood history is material to flood cover underwriting; inaccurate answers at inception permit retrospective endorsement even if made in good faith; Flood Re scheme accessible only via direct broker/insurer route, not price comparison sites; insurer must demonstrate via underwriting evidence it would not have offered cover if true facts known</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Not applicable — insurer had underwriting guidelines and government flood risk data; outcome did not depend on missing evidence</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>Ms J answered questions to best of knowledge — accepted in good faith; but inaccuracy was material regardless of intent; Ocaso provided underwriting guidelines confirming flood cover would never have been offered for this property; property classified as high flood risk by government; Ocaso instructed broker to notify Ms J promptly; Ms J confirmed she wanted policy to continue without flood cover; Flood Re unavailable via PCW channel; neighbour's circumstances unknown and irrelevant</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>Properties acquired via price comparison sites cannot access Flood Re underwriting — Flood Re eligibility requires direct broker/insurer engagement at point of sale; undisclosed prior flood history (even where policyholder is unaware) permits retrospective flood exclusion if insurer can demonstrate it would not have offered cover; good faith at inception does not prevent retrospective endorsement where misrepresentation is established</t>
+        </is>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>IF undisclosed_prior_flood_history_discovered AND insurer_underwriting_evidence_shows_cover_would_not_have_been_offered THEN flood_exclusion_endorsement_valid_retrospective_to_inception; Flood_Re NOT available IF policy_obtained_via_price_comparison_site</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2787998.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="120" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2800821</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>3 Jun 2021</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Premium pricing dispute — Aviva rated property as high flood risk from 2012 causing 73-47% annual premium increases; dispute whether 2012-2015 and 2016-2018 premiums were fair; Flood Re launched 2016 but premiums not proportionally reduced; also: 2006 claim incorrectly included causing overcharge 2014-2019 (already refunded £1,161)</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — no flood damage claim; complaint concerns premium pricing linked to high flood risk rating</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Not applicable — no flood claim was made; dispute concerns premium pricing and administration</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Aviva cited flood mapping model rating property at significant flood risk from 2012; ABI Statement of Principles 2008 as basis for continuing cover at elevated premium; Mr D disputed the flood risk rating and ability to find alternative quotes at ~£400/year; Aviva could not provide pre-2014 premium breakdown (bank administered policy until 2014); Flood Re Scheme cost was £330-335 per year for property</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Upheld in part — 2012-2015 premiums fair (flood risk rating justified per ABI Statement of Principles); 2016-2018 premiums excessive post-Flood Re cession; Aviva to recalculate 2016-2018 premiums as (2011 base premium less insurance premium tax less 10% flood loading) plus Flood Re cost plus applicable insurance premium tax; refund difference with 8% simple interest per annum from date of each instalment; 2006 claim overcharge already remedied (£1,161 refunded). Aviva must also cancel and reissue uncashed cheques if required.</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
+        <is>
+          <t>ABI Statement of Principles 2008 — insurer obligation to continue cover for existing high flood risk policyholders; Flood Re scheme (launched 2016) — flood risk cession mechanism; duty not to exploit policyholder non-engagement; insurer deemed to know policyholder is not engaging by fifth renewal (2015 for Mrs D); premium after Flood Re cession must reflect actual retained risk only</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>Pre-2014 premium breakdown unavailable (bank administered policy until 2014); proportion of 2011 premium attributable to flood risk unknown — FOS applied 10% proxy deduction in absence of true figure</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>Insurer entitled to change flood risk assessment and increase premium; ABI Statement of Principles justified continued cover at elevated premiums 2012-2015 without sudden increases (phased increases acknowledged); once Flood Re cession in 2016 transferred flood risk, retained premium should have returned to pre-risk-rating base plus Flood Re charges; residual premium still 234% above pre-2012 level despite cession; insurer exploited non-engagement after 5th renewal; 10% proxy deduction applied as equitable substitute for unknown 2011 flood loading</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>After Flood Re cession, insurers must recalibrate retained premium to exclude the flood risk element now covered by Flood Re; inflated pre-cession flood premiums cannot simply continue post-cession; policy administration handovers should audit prior claim loadings for accuracy; FOS considers an insurer ought to know a policyholder is not engaging by their fifth renewal</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>IF flood_re_cession = TRUE AND premium_not_reduced_to_reflect_ceded_flood_risk THEN investigate_post_cession_overcharge; IF policy_administration_transferred THEN audit_prior_claim_loadings_for_accuracy; IF policyholder_has_not_engaged_by_5th_renewal THEN insurer_must_not_exploit_inertia_by_above_market_increases</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2800821.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="120" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-020</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2882609</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>3 Aug 2021</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Flood claim accepted but settlement inadequate — Aviva paid £4,629.19 for drying and redecoration only; refused full structural waterproofing repairs citing betterment and wear and tear; 200-year-old stone property flooded following named storm February 2020</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>External flood water via ground floor — 200-year-old solid stone walls; external ground levels higher than internal floor in places; no damp proof course or internal tanking; water entered ground floor via wall/floor junction; property had no prior flood claim</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Residential home (200-year-old stone property with 45-year extension)</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Aviva argued full structural waterproofing and DPC works would constitute betterment — structural deficiencies (no DPC, no tanking, high external ground levels) attributed to age, wear and tear, and poor construction pre-dating the flood; settlement limited to drying out and redecoration (£4,629.19) as restoring pre-loss condition</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Aviva surveyor attributed structural deficiencies to age/wear/tear not flood — concluded drying and redecoration restored property to pre-loss condition; claimant argued property was watertight before flood (no prior claim); water re-entered after Aviva's settlement confirming inadequacy; claimant self-funded approximately £16,000 in repairs; surveyor's own comments confirmed drying/redecoration would not prevent future water ingress</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Complaint upheld — Aviva must arrange effective and long-lasting repairs to prevent future flood damage, or reimburse Mr O's repair costs with 8% simple interest per annum from date of payment; drying and redecoration insufficient as confirmed by surveyor's own evidence; once claim accepted insurer cannot rely on wear and tear exclusion to avoid paying for effective repairs; betterment principle does not apply where repairs restore (not improve) pre-loss condition</t>
+        </is>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>Indemnity principle — insurer must provide effective and long-lasting repairs, not merely cosmetic restoration; betterment does not apply where works are necessary to restore pre-loss watertight condition (not to improve upon it); once claim accepted, insurer cannot rely on wear and tear exclusion to deny effective repairs for the same claim; property built to building regulations at time of construction is assumed adequate unless pre-existing deficiency is evidenced</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>Pre-loss structural survey or DPC testing confirming property was or was not watertight before flood; independent assessment distinguishing flood-caused damage from pre-existing deficiencies; itemised repair costs for flood-attributable works vs structural improvement; no prior flood claim or water ingress evidence to support pre-existing deficiency argument</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>No prior flood claim and no evidence property was not watertight before February 2020 event; property and extension assumed built to building regulations at time; once claim accepted, insurer bound to provide effective and lasting repair; surveyor's own letter confirmed drying/redecoration would not prevent recurrence — this undermines Aviva's position; water re-entered confirming inadequacy of settlement; betterment only applies where repairs improve property beyond pre-loss state — here they merely restore it; wear and tear exclusion cannot be invoked after accepting claim to avoid liability for effective repairs</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>Betterment argument fails when property had no prior water ingress and structural works are necessary to restore pre-flood watertight condition; insurers should conduct thorough pre-settlement structural surveys to separate pre-existing deficiencies from flood-caused vulnerabilities before accepting; accepting a claim forecloses subsequent reliance on wear and tear to deny effective reinstatement; surveyor comments acknowledging inadequacy of proposed repairs are binding admissions</t>
+        </is>
+      </c>
+      <c r="T21" s="5" t="inlineStr">
+        <is>
+          <t>IF claim_accepted = TRUE AND no_prior_water_ingress_history AND surveyor_confirms_proposed_repairs_inadequate THEN insurer_must_fund_effective_lasting_repairs; betterment_exclusion NOT applicable WHERE repairs_restore_not_improve_pre_loss_condition</t>
+        </is>
+      </c>
+      <c r="U21" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2882609.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add FLOOD-021 to FLOOD-030 to Flood Case Database - Batch 3 complete
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Flood_Case_Database.xlsx
+++ b/knowledge/case-databases/Flood_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2703,6 +2703,1056 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="120" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2922192</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>St Andrew's Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Jul 2021</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Flood risk premium loading dispute — Flood Re cession; no flood damage claim; complaint about flood risk rating methodology and large annual premium increases (20% per year, 2018–2020)</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>N/A — no flood event; complaint concerns flood risk premium pricing and address-point vs postcode rating methodology</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>N/A — no claim declined; complaint about flood risk premium pricing; insurer applied address-point flood risk rating from 2015, ceded policy to Flood Re from 2016; premium increases attributed to general pricing policy changes alongside flood risk component</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Mr and Mrs W: property protected by earth flood barrier built 2009; elevated position; Flood Re website shows low-to-very-low flood risk for address; no prior flooding in 41 years. St Andrew's: uses multiple data sources including third-party flood risk models, EA data, and local authority flood maps; address-point rating from 2015 increased their flood band rating; cession to Flood Re capped flood risk element but overall premium also includes non-flood components</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — insurer entitled to use postcode or address-point flood risk rating consistently without individual property assessments; Flood Re cession correctly applied (capping flood risk element); overall premium increases since 2016 in line with general pricing policy; Mr and Mrs W were not singled out; no unfair or unreasonable treatment found</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P22" s="3" t="inlineStr">
+        <is>
+          <t>Flood Re scheme cession — flood risk premium element capped; address-point rating methodology; insurer entitled to set flood risk premiums based on its own consistent model data; FOS will not interfere with insurer's commercial pricing judgements unless clearly unfair</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>Individual property-level flood survey distinguishing this address from higher-risk neighbours in the same postcode; breakdown of non-flood vs flood premium components at each renewal</t>
+        </is>
+      </c>
+      <c r="R22" s="3" t="inlineStr">
+        <is>
+          <t>Insurer entitled to use consistent rating methodology (postcode or address-point) without individual assessment for each property — cost-prohibitive; Flood Re scheme working as designed (capping flood premium element); premium increases since 2016 reflect general pricing adjustments alongside Flood Re, not scheme misapplication; Mr and Mrs W not singled out; no right or wrong way to assess flood risk provided consistent methodology applied</t>
+        </is>
+      </c>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>Flood Re cession caps only the flood risk component of the premium — the retained premium for other risks can still increase under general pricing policy; customers may experience overall premium increases even after Flood Re cession if non-flood pricing elements rise; FOS will not challenge insurer's flood risk rating model absent clear inconsistency or unfair singling out</t>
+        </is>
+      </c>
+      <c r="T22" s="3" t="inlineStr">
+        <is>
+          <t>IF flood_re_cession = True AND customer_disputes_premium_increase THEN insurer_methodology_upheld IF consistent_with_general_pricing_policy AND no_evidence_of_unfair_singling_out; Flood_Re_cession DOES NOT guarantee reduced overall premium if non-flood retained components increase</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>DRN-2922192.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="120" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-022</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2928961</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Sep 2021</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Commercial landlord buildings insurance — claimed flash flood to shop floor on 13 August 2020; insurer declined for failure to prove insured event occurred; tenant alleged water found on shop floor during storm conditions</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>External — claimed flash flood through front of shop; insurer's surveyor found no moisture or storm-consistent damage; weather records showed only 1.6mm/hr maximum rainfall on date of incident (not storm conditions)</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Commercial (shop / retail)</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Policyholder failed to discharge burden of proving an insured event occurred — insurer's surveyor (Company B, 1 month post-incident) found no moisture in floor, no wall/skirting damage, no stock damage; weather records confirmed no storm or flood conditions on the date; no photos of flooding taken; no media reports or evidence of wider area flooding; damage attributed to long-term wear and tear and material breakdown</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Company B (insurer, 1 month post-incident): no moisture, no skirting/wall damage, floor damage = wear and tear/material breakdown. Company C (policyholder, 3 months post-incident): floor saturated, concluded flash flood cause. Weather records: 1.6mm/hr maximum — not storm conditions. FOS placed greater weight on Company B's earlier inspection and independent weather data</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — AXA's decline of the claim was fair and reasonable; policyholder did not discharge burden of proving an insured event; no contemporaneous evidence of flooding; Company B's earlier, more proximate inspection findings given greater weight than Company C's later inspection</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>Flood defined as 'escape of water from the normal confines of any natural or artificial water course, lake, reservoir, canal, drain or dam; inundation from the sea; rain induced run-off; whether resulting from storm or not'; policyholder bears burden of proving insured event occurred; earlier expert inspection given greater evidential weight</t>
+        </is>
+      </c>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>Contemporaneous photographs of flooding by tenant; weather data supporting storm or heavy rainfall on 13 August 2020; evidence of wider area flooding (media reports, neighbouring premises claims); moisture readings taken at time of incident rather than 1 or 3 months later</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>Onus on policyholder to prove insured event — not discharged here; Company B's earlier inspection (1 month post-incident) found no moisture, no skirting/wall damage consistent with flooding, and stock undamaged; weather records confirmed only 1.6mm/hr rainfall (not storm conditions); no corroborating evidence of flash flooding in area; Company C's saturated floor reading 3 months later cannot be reliably attributed to August 2020 incident; wear and tear excluded under accidental damage cover</t>
+        </is>
+      </c>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>In flood claims on commercial properties, the timing of expert inspections is critical — the longer the gap between incident and inspection, the weaker the evidential link; absence of contemporaneous photos, weather data, and corroborating area evidence makes proof of flash flood very difficult; tenant reporting water 'during storm conditions' is insufficient without corroboration where weather data contradicts storm conditions</t>
+        </is>
+      </c>
+      <c r="T23" s="5" t="inlineStr">
+        <is>
+          <t>IF flood_claim AND no_contemporaneous_evidence AND insurer_expert_inspected_earlier_than_policyholder_expert THEN weight_earlier_expert_report_more_heavily AND consider_declining_if_burden_not_discharged; absence_of_stock_damage_and_skirting_damage = negative_indicator_for_flooding</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2928961.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="120" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>DRN2955063</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Millennium Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Rented residential property — flooded by agricultural field surface water runoff during thunderstorm; insurer voided policy and declined flood claim citing non-disclosure of proximity to watercourse (130m brook) and flood risk</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>External — agricultural field surface water runoff caused by severe thunderstorm exceptional rainfall; water ran off adjacent field into street flooding numerous properties; not river overbank flooding</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Residential (rented)</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Insurer voided policy from inception citing non-disclosure — Mr A answered 'No' to questions about property being in a flood risk area and near a watercourse; a brook was located approximately 130m away; insurer concluded answers were inaccurate</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Insurer: brook 130m away = watercourse 'near' property; property in flood risk area. Mr A: questions were ambiguous ('near', 'area subject to flooding' undefined); property never previously flooded in 40+ years; neighbours confirmed no prior flooding on the road; EA flood risk data showed likelihood was 'low'; flooding was exceptional one-off event from agricultural runoff not typical flood risk. FOS agreed questions were ambiguous</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>Complaint upheld — insurer's voidance and claim decline were unreasonable; non-disclosure questions were ambiguous and not sufficiently specific to fix Mr A with liability; 'near' undefined, no specific distance given; EA data indicated 'low' flood risk; Mr A took reasonable care in answering; insurer must reinstate policy, process claim, pay £200 D&amp;I compensation, remove voidance from all databases</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P24" s="3" t="inlineStr">
+        <is>
+          <t>Insurer must ask specific and clear non-disclosure questions; undefined terms ('near', 'area subject to flooding') cannot support policy voidance; if proximity threshold is material to underwriting (e.g. within 250m), question must state that threshold; pre-CIDRA reasonable care test — insurer cannot apply strict liability for ambiguous questions; one-off exceptional rainfall causing agricultural runoff is different from inherent flood risk from nearby watercourse</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>Specific distance threshold in questions; insurer's own underwriting acceptance criteria referencing proximity to watercourses (criteria did not reference rivers/watercourses at all); EA flood risk data for the specific property address</t>
+        </is>
+      </c>
+      <c r="R24" s="3" t="inlineStr">
+        <is>
+          <t>FOS principle: onus on insurer to ask specific, clear questions; 'near' in ordinary meaning is subjective — insurer itself suggested 250m as critical but did not ask that; acceptance criteria did not reference rivers/watercourses, undermining the materiality claim; flooding caused by exceptional rainfall runoff from agricultural field — different from typical watercourse-flooding risk scenario; EA data showed 'low' flood likelihood; property never previously flooded; Mr A's answers reflected reasonable care; voidance of policy caused significant distress — £200 D&amp;I appropriate</t>
+        </is>
+      </c>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>Insurers cannot void policies based on vague proximity questions; if specific distance thresholds are material underwriting criteria (e.g. 'within 250 metres of a watercourse'), those thresholds must be stated explicitly in the question; one-off exceptional rainfall events causing surface water flooding may be categorised differently from inherent flood risk posed by adjacent watercourses; acceptance criteria should be internally consistent with questions asked</t>
+        </is>
+      </c>
+      <c r="T24" s="3" t="inlineStr">
+        <is>
+          <t>IF policy_voided_for_non_disclosure AND question_text_lacks_specific_distance_threshold AND insurer_underwriting_criteria_not_referenced_in_question THEN voidance_likely_unfair; IF flooding_from_exceptional_rainfall_runoff AND property_not_in_flood_risk_area AND no_prior_flooding THEN consider_one_off_exceptional_event_vs_inherent_risk</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>DRN2955063.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="120" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-024</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2965648</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Ocaso SA, Compania de Seguros y Reaseguros</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Aug 2021</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Residential buildings and contents — house flooded by surface water/drain overwhelm during wet storm; claim declined under CIDRA careless misrepresentation — Mr S stated home was &gt;400m from river at inception (actually within 80m); insurer retrospectively applied flood exclusion endorsement</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>External — surface water flooding from drains overwhelmed by torrential rainfall during storm; river was not the source of flooding; Mr S's property within 80m of river but river did not cause the flood</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>CIDRA careless qualifying misrepresentation — Mr S declared home was &gt;400m (and &gt;200m on statement of fact) from river; property actually within 80m; had correct distance been declared, insurer would have assessed flood risk and applied Flood Exclusion Endorsement 011 from inception; endorsement also excludes 'flood resulting from storm' blocking the storm route; 'but for' test — storm caused drain overwhelm = flood from storm = excluded</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>Mr S argued river was not the cause of the flood (surface water/drain overwhelm) so proximity misrepresentation was irrelevant; insurer argued correct proximity declaration would have triggered flood exclusion regardless of flood source; FOS agreed flood exclusion applied to all flood including from storm and was not limited to river flooding</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — CIDRA careless qualifying misrepresentation established; Mr S responsible for accuracy of proximity declarations; Ocaso entitled to apply retrospective flood exclusion under CIDRA remedy; flood exclusion covered 'flood resulting from storm' so storm route equally blocked; 'escape of water' exception in exclusion applies only to internal fixed apparatus not external public drains</t>
+        </is>
+      </c>
+      <c r="N25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>CIDRA s.4(1) careless misrepresentation remedy — insurer may treat policy as if entered on terms it would have applied without the misrepresentation; Endorsement 011 Flood Exclusion Clause: (a) watercourse escape; (b) sea inundation; (c) flood resulting from storm or tempest or any other peril except escape of water from fixed water tanks, apparatus or pipes; 'escape of water' exception covers only internal apparatus flooding, not failure of external public drainage to absorb rainfall</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>Accurate proximity declaration at inception; whether insurer's underwriting criteria would have applied a narrower river-specific exclusion (rather than a broad flood exclusion) had correct distance been disclosed</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>CIDRA careless misrepresentation established — Mr S declared property &gt;400m from river; actually within 80m; Mr S responsible for taking reasonable care regardless of whether river was visible; qualifying misrepresentation because correct declaration would have triggered flood exclusion; 'but for' test: storm caused drains to overwhelm = surface water flooding from storm = excluded under endorsement; 'escape of water' exception requires internal apparatus (tanks/pipes) not external public drains overwhelmed by rainfall volume</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>Broadly drafted flood exclusions covering 'flood resulting from storm' can simultaneously block both the flood and storm routes; 'escape of water' exception in flood exclusion clauses is narrow — covers only internal fixed water apparatus (pipes, tanks), not public drainage infrastructure; CIDRA misrepresentation allows retrospective application of terms the insurer would have used at inception even where actual flood cause was unrelated to the misrepresented fact</t>
+        </is>
+      </c>
+      <c r="T25" s="5" t="inlineStr">
+        <is>
+          <t>IF flood_exclusion_includes_flood_from_storm AND cause_is_storm_surface_water_drain_overwhelm THEN storm_route_also_blocked; IF cidra_careless_misrepresentation AND qualifying THEN insurer_may_retrospectively_apply_exclusion_terms_from_inception; escape_of_water_exception_in_flood_exclusion_does_not_cover_public_drainage_failure</t>
+        </is>
+      </c>
+      <c r="U25" s="4" t="inlineStr">
+        <is>
+          <t>DRN-2965648.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="120" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3121807</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Ocaso SA, Compania de Seguros y Reaseguros</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Nov 2021</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Residential home — August 2020 flood from torrential rainfall; local drainage overwhelmed, local dam and river burst; ~3 feet of water entered property via front door and conservatory; claim declined under comprehensive flood exclusion endorsement; policyholders argued some damage from burst pipes</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>External — dam/river burst and drainage overwhelm from torrential overnight rainfall; water entered via front door and conservatory at ground level; road outside flooded (20 houses on road confirmed flooded by news reports)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Comprehensive flood exclusion endorsement (Endorsement 011) on policy schedule excludes all flood from storm, river/dam, or watercourse escape; no evidence of burst pipes separate from flood causation; assessor attributed all damage to 3 feet of flood water entering via front door and conservatory; bursting-pipes allegation unsupported</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Mr H argued some damage caused by burst pipes (separate covered peril); insurance assessor's report and local news confirmed all 20 homes on road flooded from dam/river burst; assessor attributed damage to flood water rising to 3 feet within ground floor; no independent evidence of burst pipes distinct from flood ingress; FOS found no separate cause established</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — Endorsement 011 flood exclusion clause clearly applies to dam/storm/river flood events; assessor's report, local news, and Mr H's own account all confirm the damage was caused by flood water; no evidence of burst pipes independent of the flood; endorsement 011 covers flooding from storm, dam, or watercourse making the exclusion comprehensive</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P26" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement 011 — Flood Exclusion Clause: (A) escape from normal confines of artificial watercourse/lake/reservoir/canal/dam; (B) sea inundation; (C) flood from storm/tempest or other peril except escape from fixed water tanks/apparatus/pipes; assessor confirmation of 3 feet of water entering property at ground level via doors = classic flood event within exclusion</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>Independent evidence of burst pipes within property distinct from flood water ingress; plumber's report or inspection confirming internal pipe failure separate from external flooding</t>
+        </is>
+      </c>
+      <c r="R26" s="3" t="inlineStr">
+        <is>
+          <t>Endorsement 011 clearly listed on policy schedule and defined at page 6; torrential overnight rainfall causing drainage overflow and dam/river burst = flood event within exclusion; 20 houses on road flooded confirming scale of event; assessor confirmed water entered via front door and conservatory to 3 feet depth; this is flood ingress — not consistent with burst pipe pattern; policyholder's burst pipe allegation unsupported by any evidence; even if pipes contributed, insurer entitled to attribute damage to flood given overwhelming evidence; endorsement covers all three flood types (watercourse, sea, storm-flood)</t>
+        </is>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>Where comprehensive flood exclusion (covering all flood types) applies, policyholders cannot escape it by alleging a concurrent covered cause (burst pipes) without independent evidence; assessor's report attributing all damage to flood water is determinative; when 20 neighbouring properties confirmed flooded simultaneously, the flood cause is established beyond doubt for the purposes of applying the exclusion</t>
+        </is>
+      </c>
+      <c r="T26" s="3" t="inlineStr">
+        <is>
+          <t>IF comprehensive_flood_exclusion AND policyholder_alleges_concurrent_covered_cause THEN require_independent_expert_evidence_of_concurrent_cause; IF assessor_confirms_flood_ingress_to_significant_depth AND local_news_confirms_area_flood THEN flood_exclusion_applies_notwithstanding_alternative_cause_allegation</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3121807.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="120" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-026</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3219788</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>QIC Europe Limited</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>May 2022</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Residential buildings insurance — two flood damage claims declined: (1) February 2021 basement flood — attributed to rising water table and failed internal waterproofing system; (2) August 2021 — road outside flooded but no evidence of water entering property at ground level; both excluded under rising water table and gradual damage policy exclusions</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Groundwater — rising water table causing increased pressure on internal basement waterproofing system (both claims); August claim: confirmed road flooding but basement damage attributed to water table rise, not surface water ingress through ground floor</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Residential home (with basement)</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>February claim: independent weather data showed minimal rainfall (max 5.6mm/hr one week before incident, not flood conditions); expert reports (Company T — waterproofing specialist; Company A — water supplier) concluded rising water table caused increased ground pressure leading to waterproofing system failure (gradual); both exclusions applied (rising water table + gradual occurrence). August claim: road flood confirmed but surveyor found no evidence of surface water entering property at ground level; no skirting/door/carpet/laminate damage consistent with surface flooding; basement damage again attributed to rising water table</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>February: Policyholder's experts (Companies A and Q) attributed to heavy rainfall / surface water. Company T (QIC's waterproofing specialist) and Company A concluded rising water table most likely cause. Independent weather data: minimal February rainfall — contradicts heavy rainfall claims. August: Mr M provided photos, fire service report, newspaper article confirming road flooding; surveyor found no ground-floor damage pattern consistent with surface flooding; water damage in basement attributed to water table not surface water</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — both claims fairly declined; February: rising water table + gradual waterproofing failure = two independent exclusions; independent weather data contradicts heavy rainfall claim; QIC's expert reports more detailed and reliable than policyholder's brief, late expert reports. August: road flood confirmed but insufficient evidence that surface water entered property; surveyor found no flood-entry damage pattern; water table again most likely cause of basement damage</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P27" s="5" t="inlineStr">
+        <is>
+          <t>Flood definition: 'substantial and abnormal build-up of water from an external source'; Flood exclusions: (d) loss or damage caused by rising water table levels; (e) anything that happens gradually; failed waterproofing system due to groundwater pressure = gradual occurrence + rising water table = dual exclusion; policyholder bears burden of proving flood as cause</t>
+        </is>
+      </c>
+      <c r="Q27" s="5" t="inlineStr">
+        <is>
+          <t>Independent hydrological report distinguishing groundwater from surface water flood for February claim; contemporaneous moisture readings or photos of February flooding; evidence of ground-floor surface water damage pattern (skirting, doors, carpets) in August claim; weather data supporting heavy rainfall in February 2021 (independent data contradicted this)</t>
+        </is>
+      </c>
+      <c r="R27" s="5" t="inlineStr">
+        <is>
+          <t>February: detailed expert reports from QIC's specialists (Company T, Company S, Company C) given greater weight than brief, late reports from policyholder's experts; weather data confirmed minimal February 2021 rainfall; Company A (independent water supplier) referenced high groundwater levels (water table), not surface water; Company T concluded waterproofing failure from groundwater pressure; both rising water table and gradual occurrence exclusions applied. August: road flood undisputed; but surveyor found no damage to skirting boards, doors, carpet, or laminate — inconsistent with surface water entry at ground level; water damage in basement pattern consistent with rising water table not overhead flooding; policyholder must prove covered cause, not merely that an external flood occurred nearby</t>
+        </is>
+      </c>
+      <c r="S27" s="5" t="inlineStr">
+        <is>
+          <t>Basement flood claims require two-stage analysis: (1) did surface water enter at ground level (no skirting/door/carpet damage = negative indicator) or (2) did groundwater rise through basement structure (excluded); rising water table + gradual waterproofing failure = dual exclusion; expert timing matters — detailed early reports outweigh brief late reports; road flooding does not prove property flooding — separate evidence of entry required</t>
+        </is>
+      </c>
+      <c r="T27" s="5" t="inlineStr">
+        <is>
+          <t>IF basement_flood AND no_skirting_board_door_carpet_damage AND no_surface_water_entry_evidence THEN consider_rising_water_table_exclusion; IF waterproofing_failure AND groundwater_pressure THEN dual_exclusion_applies (rising_water_table + gradual_occurrence); confirm_external_flood_does_not_automatically_prove_property_flood_ingress</t>
+        </is>
+      </c>
+      <c r="U27" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3219788.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="120" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>DRN3290959</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Ageas Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2019</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Residential home — June 2016 excessive rain overwhelmed drains; water backed up and flooded home via submerged air bricks at ground floor; broad flood exclusion endorsement on policy; claimants argued damage was caused by storm or escape of water from fixed apparatus rather than flood</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>External — drain overwhelm from excessive rainfall; water entered property via submerged ventilation bricks (air bricks) at ground floor level; river and/or drains overflowed; several inches of standing water inside property</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Broad flood exclusion endorsement covers all flood damage except from fixed water apparatus; drain overflow from excessive rain = flood (not storm, not escape of water from apparatus); water entering via submerged air bricks = flood ingress, not apparatus escape; storm route inapplicable — damage pattern (several inches of standing water) is flood damage not typical storm damage; customer agreed to endorsement at inception; no evidence water over-spilled from bath/sink (apparatus escape route not established)</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Mr C and Mrs T: event was storm-driven rain not river flood; storm should be covered; also damage from waste/soil pipe escape indistinguishable from river water. Ageas: water coming into property from outside = flood regardless of source (river or drains); flood endorsement covers all flood. Photos: no evidence of bath/sink overflows; air bricks at ground floor level submerged by external flood water. FOS: confirmed water entering via submerged air bricks = flood not apparatus escape</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — flood endorsement is clearly worded and broadly applies to all flood; water entering via submerged air bricks from external floodwater = flood, not escape from fixed apparatus; storm damage requires storm-type evidence (tiles, staining) not several inches of standing water; emergency strip-out by insurer's agents simultaneously with cover warnings did not constitute acceptance of cover; endorsement fairly applied</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
+        <is>
+          <t>Broad flood exclusion endorsement: 'does not cover loss or damage caused by flood other than directly resulting from escape of water from fixed water tanks, apparatus or pipes'; flood = body or mass of water appearing where it should not be, regardless of cause (river or drain overflow); storm damage = tiles missing, staining/dampness — not several inches of standing water; emergency insurer response ≠ acceptance of cover; endorsement agreed at inception</t>
+        </is>
+      </c>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>Evidence that waste/soil pipes within property overflowed independently of the external flood (photos from during flood showed no bath/sink overflows); loss adjuster's July 2017 report identified air bricks as flood entry point</t>
+        </is>
+      </c>
+      <c r="R28" s="3" t="inlineStr">
+        <is>
+          <t>Flood endorsement is clear — Mr C accepted it, even if he misunderstood its scope; endorsement covers all flood except from fixed water apparatus (escape of water exception); water entering via submerged air bricks is external flood ingress, not apparatus escape; storm cover requires damage typical of storms (tiles, water staining) — not several inches of standing water which is flood-type damage; insurer's emergency strip-out response was appropriate emergency action not cover acceptance, given simultaneous warnings about cover doubts and formal decline within a fortnight; no evidence waste/soil pipes independently overflowed — photos show no overflowing fixtures</t>
+        </is>
+      </c>
+      <c r="S28" s="3" t="inlineStr">
+        <is>
+          <t>When insurer deploys emergency contractors before confirming liability, always issue simultaneous written warnings that emergency response does not constitute cover acceptance; broad flood exclusion endorsement overrides both storm and escape-of-water routes if damage pattern is flooding (standing water); water entering via submerged air/ventilation bricks is flood ingress, not escape of water from apparatus</t>
+        </is>
+      </c>
+      <c r="T28" s="3" t="inlineStr">
+        <is>
+          <t>IF flood_exclusion_endorsement_agreed_at_inception AND water_entered_via_submerged_air_bricks THEN escape_of_water_from_apparatus_exception_does_not_apply; IF insurer_deploys_emergency_contractors AND exclusion_flagged_simultaneously THEN emergency_response_not_cover_acceptance; storm_damage_requires_storm_type_evidence_not_standing_water_pattern</t>
+        </is>
+      </c>
+      <c r="U28" s="2" t="inlineStr">
+        <is>
+          <t>DRN3290959.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="120" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-028</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3295916</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>QIC Europe Ltd</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Apr 2022</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Residential home — August 2020 flood claim; QIC voided policy back to 2019 alleging failure to declare 2018 'flood' at renewal; 2018 incident was public drain overflow onto pavement/gravel at front of property — no damage to property, water soaked into gravel and disappeared; CIDRA reasonable consumer test</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>External — August 2020 actual flood at property; 2018 alleged prior flood was a transient public drain overflow during heavy rain: water flowed across public footpath, entered gravel at front of property, soaked in, disappeared — no entry to property, no property damage</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>QIC: 2018 drain overflow technically meets policy definition of flood ('substantial and abnormal build-up of water from an external source'); Mr H should have declared it at 2019 renewal (statement of fact said property not affected by flood in last 10 years); QIC would not have renewed if known; careless CIDRA misrepresentation; avoided policy back to 2019 and declined 2020 claim</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>QIC: any external water overflow onto property = declarable flood regardless of scale. Mr H: described 2018 incident honestly — water overflowed public drain onto pavement, soaked into front garden gravel, no property entry, no damage, brief and fleeting; normal consumers would not see this as a flood requiring declaration. FOS: CIDRA test is reasonable consumer standard, not strict policy definition; brief drain overflow with no property damage not declarable by reasonable consumer</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>Complaint upheld — CIDRA reasonable consumer standard applies, not strict policy definition; fleeting drain overflow on public footpath with no property entry or damage is not what a reasonable consumer would consider a declarable flood; QIC's policy avoidance was unfair and outside CIDRA entitlement; QIC to: pay 2020 flood claim in full (less excess and any premium refunds) including alternative accommodation, disturbance allowance, travel expenses, utility bills, and out-of-pocket expenses; 8% simple interest on settlement from claim date to offer date; £1,000 D&amp;I compensation; remove void record from QIC files and CUE database</t>
+        </is>
+      </c>
+      <c r="N29" s="4" t="n">
+        <v>1000</v>
+      </c>
+      <c r="O29" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P29" s="5" t="inlineStr">
+        <is>
+          <t>CIDRA — standard of care is that of a reasonable consumer; QIC renewal statement of fact: 'property or any property within 100m has NOT been affected by flood within the last 10 years'; test is what a reasonable consumer would deem declarable, not the strict policy definition of flood; brief transient public drain overflow with no property damage not declarable by reasonable consumer standard</t>
+        </is>
+      </c>
+      <c r="Q29" s="5" t="inlineStr">
+        <is>
+          <t>QIC had no evidence the 2018 incident was known as a flood event locally or caused damage; Mr H's consistent honest account (including knowing QIC would categorise it as a flood) supported credibility; no evidence Mr H was downplaying the 2018 incident</t>
+        </is>
+      </c>
+      <c r="R29" s="5" t="inlineStr">
+        <is>
+          <t>CIDRA test = reasonable consumer standard, not policy definition; Mr H honestly described 2018 incident — water flowed across public footpath into gravel, soaked in, no property entry, no damage, disappeared quickly during 30-minute heavy rain; this is the kind of transient drain overflow commonly experienced during sudden heavy rain across UK streets — reasonable consumer would not consider this a flood requiring insurance declaration; Mr H's honesty in acknowledging the incident while contesting its characterisation weighs in his favour; QIC's strict definitional approach misapplied CIDRA; substantial financial and personal impact on family (COVID key worker; two sets of living costs; stress diagnosis) justified £1,000 D&amp;I</t>
+        </is>
+      </c>
+      <c r="S29" s="5" t="inlineStr">
+        <is>
+          <t>Insurers cannot apply strict policy definitions of 'flood' to defeat CIDRA's reasonable consumer standard in non-disclosure avoidance cases; a transient drain overflow with no property damage is not a declarable flood by reasonable consumer standards; asking courts to characterise minor, fleeting water incidents as prior floods for avoidance purposes is unlikely to succeed under CIDRA; policy avoidance has severe collateral consequences (CUE record, claim decline, two households to fund) that FOS weighs in setting D&amp;I quantum</t>
+        </is>
+      </c>
+      <c r="T29" s="5" t="inlineStr">
+        <is>
+          <t>IF cidra_non_disclosure AND prior_incident_is_fleeting_drain_overflow AND no_property_damage AND no_property_entry THEN reasonable_consumer_would_not_declare; apply_cidra_reasonable_consumer_test_not_strict_policy_definition_to_non_disclosure_avoidance; IF policy_voided_AND_severe_personal_financial_impact THEN higher_d_and_i_quantum_warranted</t>
+        </is>
+      </c>
+      <c r="U29" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3295916.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="120" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>DRN3348419</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Jul 2016</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Commercial business property — secondary latent damage claim; RSA accepted and settled 2007 flood claim; in 2015 Mr W claimed further damage (pool table flooring, cellar, car park, paving/tree, cellar stairs floor) allegedly caused by the same 2007 flood; RSA declined the supplementary claim</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>External — original 2007 flood (insured event accepted); secondary claim for latent moisture damage discovered years later including adhesive failure in pool table flooring area and potential cellar/car park damage</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Commercial (public house / business premises)</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>RSA disputed that most secondary damage areas (cellar, car park, paving/tree, cellar stairs) were caused by the 2007 flood; insufficient expert evidence linking these areas to the flood; only pool table flooring area had sufficient evidence of flood causation; cellar damage negated by damp specialist; car park cause unclear per structural engineer; no expert opinion on paving/tree or cellar stairs</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Structural engineer: car park cause unclear, cannot link to flood; cellar may have been affected; pool table floor adhesive failed due to moisture. Damp specialist: cellar damage unlikely caused by flood. Flooring specialist: water got between vinyl and floor around pool table = adhesive degraded. No expert opinion on paving/tree or cellar stairs floor. Adjudicator and FOS agreed pool table area proven; cellar stairs to be inspected; all other areas insufficient evidence</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>Complaint upheld in part — RSA to pay £5,000 for pool table area floor and ceiling repair (evidentially linked to 2007 flood via structural engineer and flooring specialist); RSA to arrange inspection of cellar stairs floor and carry out repairs if flood-caused; all other areas (cellar, car park, paving/tree) not proven as flood-caused; RSA's £5,000 cash offer reasonable given re-carpeting cost ~£4,000</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>Policyholder bears burden of proof for each claimed area of damage; secondary flood damage claims years after original accepted claim require area-specific expert evidence linking damage to the original insured event; flood causation assessed separately for each area of claim; FOS will disaggregate multi-area claims and assess evidential basis for each element individually</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>Expert opinion on paving/tree and cellar stairs floor (no expert report for these areas); independent survey of cellar (damp specialist later negated claim after adjudicator recommendation); stronger pre-loss condition evidence for car park area</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="inlineStr">
+        <is>
+          <t>Each area of claimed damage assessed against expert evidence available: pool table flooring confirmed via structural engineer (moisture causing adhesive failure) and flooring specialist (water between vinyl and floor); cellar: damp specialist concluded unlikely to be flood-caused; car park: structural engineer could not determine flood causation; paving/tree and cellar stairs: no expert opinion at all; policyholder's burden not discharged for unsubstantiated areas; £5,000 RSA offer reasonable vs re-carpeting cost of ~£4,000; cellar stairs floor to be inspected as outstanding area of uncertainty</t>
+        </is>
+      </c>
+      <c r="S30" s="3" t="inlineStr">
+        <is>
+          <t>Secondary flood damage claims made years after the original event require separate expert reports for each claimed area — global claims without area-specific causation evidence will be disaggregated and rejected for unsubstantiated areas; FOS will assess each area independently; the original claim acceptance does not extend to subsequently discovered damage without individual expert linkage to the original flood event</t>
+        </is>
+      </c>
+      <c r="T30" s="3" t="inlineStr">
+        <is>
+          <t>IF secondary_flood_damage_claim AND years_after_original_accepted_event THEN require_separate_expert_causation_evidence_per_claimed_area; IF claim_partially_proven THEN partial_settlement_ordered_for_proven_areas_only; original_claim_acceptance_does_not_automatically_cover_latent_damage_discovered_later</t>
+        </is>
+      </c>
+      <c r="U30" s="2" t="inlineStr">
+        <is>
+          <t>DRN3348419.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="120" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-030</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3370157</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Fairmead Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Apr 2022</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>No flood claim made — complaint about policy ambiguity regarding scope of flood cover; Mr and Mrs T live in flood zone and sought confirmation that policy would cover a future flood; alleged mis-sale; Fairmead failed to respond to written queries</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no flood event; complaint concerns policy wording clarity and insurer's obligation to pre-confirm flood cover</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no flood claim declined; complaint about policy wording ambiguity; Fairmead confirmed flood is an insured peril but could not give blanket pre-confirmation that all future flood claims would be covered (exclusions must be applied on a claim-by-claim basis)</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>Mr and Mrs T: policy says covered for 'flood' but also excludes 'water entering the building' under Accidental Damage and 'underground water' under flood cover — contradictory and misleading; also verbal assurance of flood cover at inception. Fairmead: policy has flood cover; 'water entering from external source' exclusion is in Accidental Damage section only, not main flood cover section; 'underground water/rising groundwater' exclusion is standard and clearly worded. FOS: no contradiction — exclusions are section-specific</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — policy does have flood cover; 'water entering from external source' exclusion applies only under the Accidental Damage section, not the main flood cover; 'underground water' exclusion is a standard and clearly worded flood cover exclusion; no insurer can give pre-confirmation that all future claims under any peril will be accepted (exclusions apply on a claim-by-claim basis); mild failing in Fairmead not responding to written queries promptly but no substantive wrongdoing; mis-sale allegation not established</t>
+        </is>
+      </c>
+      <c r="N31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P31" s="5" t="inlineStr">
+        <is>
+          <t>Policy flood cover: buildings and contents covered against flood as standard peril; Accidental Damage exclusion for 'damage caused by water entering the buildings from an external source' — applies to AD section only, not main flood cover; flood cover exclusion for 'underground water/rising groundwater' — standard exclusion; no insurer can pre-confirm coverage for all future claims without knowing the circumstances</t>
+        </is>
+      </c>
+      <c r="Q31" s="5" t="inlineStr">
+        <is>
+          <t>N/A — complaint was about policy interpretation, not a live flood claim with disputed evidence</t>
+        </is>
+      </c>
+      <c r="R31" s="5" t="inlineStr">
+        <is>
+          <t>Policy has flood cover as an insured peril — this was correctly communicated at inception; 'water entering from external source' exclusion is limited to the Accidental Damage section of the policy, not the main flood cover — the two sections are different and independent; rising groundwater exclusion under flood cover is standard and clearly worded; no insurer can give blanket pre-confirmation about future claims as exclusions must be assessed on the facts of each claim; initial verbal assurance of 'flood cover' was accurate (policy does have flood cover); Fairmead's failure to respond promptly to written queries is a minor administrative failing but not substantive unfairness</t>
+        </is>
+      </c>
+      <c r="S31" s="5" t="inlineStr">
+        <is>
+          <t>Policy documents with multiple sections (main peril cover; accidental damage; exclusions) may appear contradictory to consumers who read them linearly — advisers should proactively explain that AD exclusions operate in a separate context from main peril cover; no insurer can pre-confirm all future flood claims will be paid without knowing the claim circumstances; rising groundwater exclusion under the flood cover section is distinct from the main flood peril cover</t>
+        </is>
+      </c>
+      <c r="T31" s="5" t="inlineStr">
+        <is>
+          <t>IF accidental_damage_exclusion_for_water_entry AND separate_main_flood_cover_exists THEN exclusion_is_section_specific_not_global; IF consumer_queries_policy_ambiguity_about_flood THEN explain_difference_between_ad_section_and_main_flood_cover; rising_groundwater_exclusion_under_flood_section_is_standard_and_enforceable</t>
+        </is>
+      </c>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>DRN-3370157.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add FLOOD-032 to FLOOD-040 to Flood Case Database - Batch 4 complete
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Flood_Case_Database.xlsx
+++ b/knowledge/case-databases/Flood_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:U40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3753,6 +3753,951 @@
         </is>
       </c>
     </row>
+    <row r="32" ht="120" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-032</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3710798</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2023</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Flood — residential; dispute about handling quality and scope of second flood repair liability; original flood claim accepted; dispute concerns whether temporary repairs were communicated as interim only, and whether second flood flooring damage was attributable to Lloyd's failure to communicate interim repair status</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>External flood (source not specified in decision — residential flood event; property flooded twice)</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>N/A — original flood claim accepted; Lloyd's disputed liability for second flood flooring damage and whether first repairs were described as permanent or temporary</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Mr D and Ms R: Lloyd's told them initial repairs were permanent; would have taken steps to prevent second flood if advised repairs were temporary. Lloyd's: repairs were temporary pending building warranty resolution; second flood not attributable to Lloyd's. FOS: even if repairs were temporary, warranty repairs would not have been completed before second flood regardless — second flood not Lloyd's fault; but Lloyd's failed to communicate interim repair nature clearly</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Lloyd's to pay £1,500 D&amp;I compensation for delay and poor communication about interim nature of repairs; Lloyd's to cover cost of flooring damaged by second flood if not covered by building warranty provider</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P32" s="3" t="inlineStr">
+        <is>
+          <t>Insurer's duty to clearly communicate when flood repairs are temporary or interim; scope of liability for damage from second flood event; building warranty exclusion does not eliminate insurer liability for repair-related communication failures; insurer bears consequential liability only to extent not recoverable from another source</t>
+        </is>
+      </c>
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>Evidence from policyholders confirming second flood flooring damage is not covered by building warranty</t>
+        </is>
+      </c>
+      <c r="R32" s="3" t="inlineStr">
+        <is>
+          <t>Lloyd's acknowledged delay and poor communication. Even if first repairs were temporary, building warranty repairs would not have been completed before second flood — so second flood would have happened regardless. Lloyd's not responsible for warranty provider failings. However, Lloyd's should pay for any flooring from second flood not covered by warranty. £1,500 compensation fair for delay and failure to explain temporary repair nature.</t>
+        </is>
+      </c>
+      <c r="S32" s="3" t="inlineStr">
+        <is>
+          <t>When insurer installs temporary flood repairs, it must explicitly communicate in writing that repairs are interim-only. Failure to do so creates legitimate expectation of permanence and potential liability for consequential second-event damage. Award scope is limited to damage not covered by any other route (e.g. building warranty).</t>
+        </is>
+      </c>
+      <c r="T32" s="3" t="inlineStr">
+        <is>
+          <t>IF temporary_flood_repairs_installed AND insurer_fails_to_communicate_interim_nature THEN partial_liability_for_second_event_damage; IF second_flood_damage AND other_coverage_available THEN insurer_liable_for_uncovered_residue_only; delay_plus_communication_failure = D_and_I_award_warranted</t>
+        </is>
+      </c>
+      <c r="U32" s="2" t="inlineStr">
+        <is>
+          <t>DRN-3710798.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="120" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-033</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>DRN4280012</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Liverpool Victoria Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Jul 2017</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Commercial buildings and business interruption insurance — severe storm caused flooding at business premises; LV declined under flood exclusion clause introduced at policy renewal in 2016; policyholder argued storm was proximate cause of damage not flood</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>External — surface water accumulation from storm; rainwater accumulated on street, drains overwhelmed, water entered premises at ground level</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Commercial (business premises)</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>Flood exclusion clause: Material Damage All Risks excludes damage arising from or in connection with flood. Loss adjuster confirmed rainwater accumulated on street until drains overwhelmed and water entered premises — flood was the proximate cause; storm was indirect cause only. Exclusion properly communicated at renewal (highlighted in red in renewal letter; separate broker email).</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>Mr D: local drains blocked by storm; storm was proximate cause; flood exclusion added at renewal without sufficient notice to broker. LV: loss adjuster report confirms surface water accumulation = flood as proximate cause; flood exclusion highlighted in red in renewal letter; broker emailed separately; broker confirmed acceptance. FOS: no expert evidence to contradict loss adjuster; flood exclusion properly communicated.</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — flood was proximate cause; storm was indirect cause only; flood exclusion properly introduced at renewal and communicated to broker; LV entitled to decline claim</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P33" s="5" t="inlineStr">
+        <is>
+          <t>Flood exclusion: Material Damage All Risks excludes damage arising from or in connection with flood; proximate cause doctrine — immediate cause of damage determines the applicable peril; insurer entitled to add flood exclusion at renewal based on updated flood mapping with proper broker notification</t>
+        </is>
+      </c>
+      <c r="Q33" s="5" t="inlineStr">
+        <is>
+          <t>N/A — loss adjuster report conclusive; no expert evidence contradicting proximate cause finding</t>
+        </is>
+      </c>
+      <c r="R33" s="5" t="inlineStr">
+        <is>
+          <t>Loss adjuster report clear: rainwater accumulated on street and rose until drains overwhelmed then entered premises = flood as direct cause; storm = indirect trigger only. No expert evidence to the contrary. Flood exclusion highlighted in red on renewal letter page 1; broker separately emailed; broker confirmed acceptance on Mr D's behalf. LV not required to notify Mr D separately once broker notified and accepted.</t>
+        </is>
+      </c>
+      <c r="S33" s="5" t="inlineStr">
+        <is>
+          <t>Proximate cause of damage is the peril that determines coverage even where a second peril (storm) triggered the chain of events. Surface water that accumulates and enters premises via overwhelmed drains = flood, not storm. Flood exclusion introduced at renewal is binding where communicated to broker in writing with clear highlighting and confirmed acceptance.</t>
+        </is>
+      </c>
+      <c r="T33" s="5" t="inlineStr">
+        <is>
+          <t>IF loss_adjuster_confirms_surface_water_accumulation_before_property_entry THEN proximate_cause_is_flood; IF flood_exclusion_highlighted_in_renewal_letter AND broker_confirmed_acceptance THEN exclusion_is_binding; storm_triggering_drain_overwhelm_is_indirect_cause_only</t>
+        </is>
+      </c>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
+          <t>DRN4280012.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="120" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-034</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>DRN4396587</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Legal &amp; General Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Apr 2020</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Residential home buildings insurance — storm and flash flooding damaged rear garden wall; L&amp;G settled as flood claim; Mr S disputed peril classification, wanted storm recorded to avoid flood claim history and future premium impact; L&amp;G also erroneously stated property is not a flood risk</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>External — surface water runoff from flash flooding during storm; water ran under property and damaged rear garden wall at or below ground level</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Peril Classification Dispute</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>N/A — claim was settled; dispute only concerns peril classification (flood vs storm) and impact on future premium declarations</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Mr S: heavy rainfall during storm caused damage directly = storm claim; if recorded as flood he would have withdrawn the claim had he known. L&amp;G: rainfall caused water to accumulate at ground level and flood = flood is proximate cause; insurer determines final peril classification, not loss adjuster. L&amp;G error: incorrectly told Mr S property is not considered a flood risk. FOS: L&amp;G correctly recorded as flood; but error re flood risk status warrants £100 compensation.</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>Flood classification upheld as correct; L&amp;G to pay £100 compensation for incorrectly informing Mr S his property is not considered a flood risk when it is</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P34" s="3" t="inlineStr">
+        <is>
+          <t>L&amp;G flood definition: water from any external source entering a building at or below ground level with substantial or abnormal volume; flood does not have to enter the building to constitute a flood event — external structures at ground level (garden walls) included; insurers determine peril classification, not loss adjustors; garden walls are buildings</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>N/A — peril classification clear from facts; flood risk status established from L&amp;G's own records</t>
+        </is>
+      </c>
+      <c r="R34" s="3" t="inlineStr">
+        <is>
+          <t>Storm rainfall caused water to accumulate and flood at ground level; accumulated flood water damaged garden wall = flood peril. If storm had caused roof damage directly, that would be storm. Peril = immediate cause of damage. Loss adjuster categorised as storm/flood preliminary; L&amp;G as insurer made final call as flood — within its authority. L&amp;G error: told Mr S property not a flood risk when it is; this incorrect information creates future insurer declaration problems for Mr S = £100 loss of expectation.</t>
+        </is>
+      </c>
+      <c r="S34" s="3" t="inlineStr">
+        <is>
+          <t>Peril classification is determined by the immediate cause of damage: accumulated flood water causing structural damage = flood, even where storm triggered the rainfall. Insurers must accurately communicate the flood risk status of a property after recording a flood claim, as this affects future declarations. A flood need not enter a building to be a flood event — flood claims include external structures (garden walls, boundary walls) at ground level.</t>
+        </is>
+      </c>
+      <c r="T34" s="3" t="inlineStr">
+        <is>
+          <t>IF storm_triggers_accumulation AND flood_water_directly_causes_damage THEN peril_is_flood_not_storm; IF insurer_records_flood_claim AND incorrectly_denies_flood_risk_status THEN compensation_for_loss_of_expectation; flood_event_does_not_require_property_entry — external_structural_damage_at_ground_level_qualifies</t>
+        </is>
+      </c>
+      <c r="U34" s="2" t="inlineStr">
+        <is>
+          <t>DRN4396587.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="120" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-035</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4415847</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Wakam</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Dec 2023</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Residential home insurance — water ingress from defective gutter on adjoining neighbour's porch canopy caused damp, bubbling plasterwork and crumbling plaster in living room; no storm; Wakam declined citing damage not caused by storm, flood, or accidental damage as defined</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Neighbour's canopy gutter overflow — defective gutter on adjoining neighbour's porch canopy abutting Ms K's property directed water into her wall</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>Wakam: no storm in area (confirmed by weather data); water from neighbour's canopy is not an overflow of external water sources as defined in policy (rivers, lakes, sea); not accidental damage (Ms K and family not the cause; damage gradual not sudden). Policy exclusion: water entering by any means other than storm or flood not covered.</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>Wakam: policy flood definition 'overflow of external water sources, such as rivers, lakes, and the sea' is exhaustive and excludes canopy ingress. Ms K: 'such as' is non-exhaustive and merely illustrative; neighbour's canopy is an external water source; contra proferentem applies. FOS: agreed with Ms K — 'such as' creates non-exhaustive list; canopy is an external water source; ambiguity resolved in policyholder's favour.</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>Complaint upheld — water ingress from neighbour's canopy falls within policy flood definition under non-exhaustive 'such as' reading and contra proferentem principle; Wakam to settle claim per remaining policy terms including any excess; £100 D&amp;I for unfair decline</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P35" s="5" t="inlineStr">
+        <is>
+          <t>Flood definition: 'overflow of external water sources, such as rivers, lakes, and the sea' — 'such as' renders source list illustrative and non-exhaustive; contra proferentem — ambiguous policy wording interpreted against insurer/drafter in policyholder's favour; accidental damage definition limited to damage caused by policyholder or family. See flood-source-of-water-interpretation.md for full analysis.</t>
+        </is>
+      </c>
+      <c r="Q35" s="5" t="inlineStr">
+        <is>
+          <t>Weather data confirming no storm (accepted by both parties); specialist report on cause of ingress from neighbour's canopy (accepted by both parties)</t>
+        </is>
+      </c>
+      <c r="R35" s="5" t="inlineStr">
+        <is>
+          <t>No storm in area — storm section does not apply. Accidental damage requires Ms K or family to have caused it — they did not. On flood: 'such as' before list of sources means list is illustrative not exhaustive. Neighbour's canopy is clearly external, clearly water-producing, clearly a source. Even if ambiguous, contra proferentem requires interpretation in policyholder's favour where insurer drafted the policy. Damage from canopy ingress = flood under policy definition.</t>
+        </is>
+      </c>
+      <c r="S35" s="5" t="inlineStr">
+        <is>
+          <t>Policy flood definitions using 'such as' before listed water sources create non-exhaustive illustrative lists — any above-ground external water source may qualify. Water ingressing from any neighbouring property structure can constitute flood where it builds up and enters the property. Where policy definition is ambiguous (source not defined), insurer cannot rely on narrow reading — contra proferentem resolves in policyholder's favour. See FLOOD-038 for contrast: rising water table (subsoil) does not qualify under same language.</t>
+        </is>
+      </c>
+      <c r="T35" s="5" t="inlineStr">
+        <is>
+          <t>IF flood_definition_uses_such_as_before_source_list THEN list_is_non_exhaustive; IF water_source_is_external_and_above_ground THEN may_qualify_as_flood_source; IF policy_wording_ambiguous THEN apply_contra_proferentem_in_policyholder_favour; distinguish_above_ground_external_overflow_from_naturally_occurring_subsoil_water</t>
+        </is>
+      </c>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4415847.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="120" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-036</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4895575</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Aug 2024</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Residential buildings and contents insurance — handling dispute; original October 2019 and February 2020 flood claims accepted; AXA withheld payment for specific 2020 flood contents items (sauna, red light therapy unit, two vibro plates, hot tub, summerhouse) invoking fraud condition; fraud condition applicability decided under separate DRN reference</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>External flood — river or surface water; property flooded October 2019 and February 2020; January 2021 flood addressed separately under DRN-4901901</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>AXA invoked fraud condition to withhold payment for specific 2020 flood items; fraud condition applicability determined unfavourable to AXA under separate complaint reference; AXA had no specific fraud concerns relating to the items in this decision</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>AXA: fraud condition entitles it to decline all three flood claims; items not paid due to wider fraud concerns. Ms G: items existed and were damaged; AXA's own fraud condition challenge was decided against AXA separately. FOS: fraud condition inapplicable (decided separately); no dispute items existed and were damaged; AXA must settle at current market rates due to delay within its own control.</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>AXA to settle claim for sauna, red light therapy unit and collagen canopy, two vibro plates, hot tub and summerhouse damaged in 2020 flood at current market rates; no D&amp;I compensation awarded as Ms G requested FOS not assess service or delay issues (pursuing separately)</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P36" s="3" t="inlineStr">
+        <is>
+          <t>Fraud condition does not apply where insurer cannot show knowing falsehood (determined separately); insurer's delay in settling accepted flood claim items means settlement at current market rates — insurer bears inflation risk for withheld payments; visitor items covered by policy but payable to visitor not policyholder</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="inlineStr">
+        <is>
+          <t>Current market rate quotes for specialist items (sauna, hot tub, summerhouse) needed to quantify settlement</t>
+        </is>
+      </c>
+      <c r="R36" s="3" t="inlineStr">
+        <is>
+          <t>No dispute that items existed and were damaged in 2020 flood. AXA provisionally accounted for costs but never paid due to fraud hold. Fraud condition decided inapplicable under separate reference. AXA had control over timing of payment and chose not to pay — must now settle at current (inflated) market rates. Ms G asked FOS not to consider D&amp;I or service quality issues — no compensation awarded in this decision.</t>
+        </is>
+      </c>
+      <c r="S36" s="3" t="inlineStr">
+        <is>
+          <t>Insurer that withholds payment for accepted flood claim items by invoking fraud condition bears the cost of price inflation if fraud condition later found inapplicable — settlement at current market rates not original claim value. Where policyholder explicitly limits scope of FOS complaint (excluding D&amp;I), FOS will not award compensation beyond what was requested. Related flood claims from same property and period may be split across multiple FOS references, each with separate award limits.</t>
+        </is>
+      </c>
+      <c r="T36" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_withholds_payment_invoking_fraud_condition AND fraud_condition_found_inapplicable THEN settle_at_current_market_rates; IF policyholder_excludes_D_and_I_from_FOS_scope THEN no_compensation_awarded; multiple_floods_same_property = separate_complaint_references_and_separate_award_limits</t>
+        </is>
+      </c>
+      <c r="U36" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4895575.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="120" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-037</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4901901</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>AXA Insurance UK Plc</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Aug 2024</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Residential buildings and contents insurance — January 2021 flood (third flood at property after 2019 and 2020 events); AXA refused to pay 2021 contents claim invoking fraud condition, alleging knowingly false statement about oil contamination in floodwater and exaggerated losses</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>External flood — river or surface water; January 2021; floodwater reportedly contaminated with oil from neighbouring property heating oil leak into local storm drains</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>AXA: fraud condition — Ms G made knowingly false statement about oil contamination (specialist found no residual oil 6 days post-flood); exaggerated losses given short interval between three flood claims and volume of items claimed; Ms G irresponsibly stored items at low level knowing flood risk. FOS: honest recollection defeats knowing falsehood; oil contamination corroborated by neighbours; AXA agent generated BER list not Ms G; reasonable for Ms G to live and store items at property.</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>AXA: specialist test 6 days post-flood found no oil = Ms G lied about oil; photo shows small initial loss report inconsistent with large final claim. Ms G: honest belief in oil contamination (smell and visual); neighbours corroborated oil in local storm drains; she explained items removed from multiple exits not just area shown in photo; items replaced after prior floods are normal day-to-day items. FOS: honest recollection standard applies; AXA agent's own BER decisions cannot found fraud; low-value items do not require individual receipts.</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>AXA cannot rely on fraud condition to refuse 2021 contents claim; must deal with claim per remaining policy terms; simple interest at 8% per annum on payment from date of initial BER report to date of payment</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P37" s="5" t="inlineStr">
+        <is>
+          <t>Fraud condition: requires knowing false statement or knowingly exaggerated claim; honest contemporaneous belief defeats fraud allegation even if later evidence contradicts it; insurer's agent decisions on BER scope are insurer's responsibility not policyholder's; low-value everyday items do not require strict proof of purchase; 8% simple interest applies where insurer has wrongly withheld payment</t>
+        </is>
+      </c>
+      <c r="Q37" s="5" t="inlineStr">
+        <is>
+          <t>Contemporaneous oil contamination evidence (sampling at time of flood rather than 6 days later); oil may have dissipated due to heavy rain in intervening period (neighbours described this pattern)</t>
+        </is>
+      </c>
+      <c r="R37" s="5" t="inlineStr">
+        <is>
+          <t>Fraud requires knowing falsehood — not established. Ms G honestly believed oil was present (smell and visual); neighbours corroborated oil in local drains and heating oil leak from neighbouring property; declining oil levels explained by heavy rain. AXA agent generated BER list and cross-referenced Ms G's list to save time — errors in that list are agent's responsibility. Policyholder with severely limited upstairs space must keep some items downstairs; not negligent. Multiple low-value items do not require individual receipts. No evidence of intentional exaggeration.</t>
+        </is>
+      </c>
+      <c r="S37" s="5" t="inlineStr">
+        <is>
+          <t>Flood fraud allegations must clear a high bar: insurer must show knowing false statement, not merely subsequent evidence of inaccuracy. Honest contemporaneous belief — especially where corroborated by neighbours — defeats fraud condition invocation. Agent-prepared BER lists that overstate or misclassify items are the insurer's own procedural error, not policyholder fraud. Policyholders living in partly-habitable flood-damaged properties cannot be required to store all items off-floor on the assumption of re-flooding.</t>
+        </is>
+      </c>
+      <c r="T37" s="5" t="inlineStr">
+        <is>
+          <t>IF fraud_condition AND alleged_false_statement AND honest_contemporaneous_belief_corroborated THEN fraud_not_established; IF agent_prepares_BER_list AND errors_in_list THEN insurer_bears_responsibility_not_policyholder; low_value_everyday_items_do_not_require_strict_receipts; IF property_partially_habitable_post_flood THEN storage_of_items_at_low_level_is_not_negligence</t>
+        </is>
+      </c>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>DRN-4901901.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="120" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-038</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4948332</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2025</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Residential home insurance (Flood Re risk) — February 2024 discovery of standing water under reception room floor; joists rotting; damage to walls; damp specialist concluded groundwater flooding from elevated water table; Aviva declined citing flood definition excludes groundwater and damage occurred gradually</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Groundwater — rising water table; standing water discovered under floor from elevated water table level possibly linked to proximity to river</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Aviva flood definition: storm or flood from overflow of external water sources, such as rivers, lakes and the sea — this does not cover groundwater or rising water table. Aviva also relied on general exclusion for damage occurring gradually. Water table is naturally occurring subsoil water that rises — not an overflow of a surface water source.</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Mrs and Mr S: groundwater flooding is an overflow of the water table which should be covered; policy wording not sufficiently clear; water in ground likely came from river exceeding its banks and saturating soil. Aviva: water table is subsoil water — not an external surface water source overflowing. Local authority and damp specialist confirmed elevated water table as cause. FOS: agreed with Aviva; water table physically distinct from surface water overflow; indirect river causation excluded in any event.</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld — groundwater from rising water table is not an overflow of external water sources as defined; Aviva's flood definition clearly distinguishes surface water overflow from subsoil groundwater; Flood Re cession does not alter peril coverage scope; Aviva acted correctly in declining claim</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P38" s="3" t="inlineStr">
+        <is>
+          <t>Flood definition: storm or flood from overflow of external water sources, such as rivers, lakes and the sea — surface overflow mechanism required; water table is naturally occurring subsoil water, not a surface overflow source; gradual damage exclusion; Flood Re scheme cession does not broaden peril coverage. See flood-source-of-water-interpretation.md for full analysis.</t>
+        </is>
+      </c>
+      <c r="Q38" s="3" t="inlineStr">
+        <is>
+          <t>N/A — cause confirmed by damp specialist and local authority as groundwater or water table; no factual dispute about cause</t>
+        </is>
+      </c>
+      <c r="R38" s="3" t="inlineStr">
+        <is>
+          <t>Policy flood definition describes surface water sources that overflow at ground level (rivers, lakes, sea) — these overflow downward causing flooding. Water table is naturally occurring subsoil water that rises upward through soil — physically and mechanically distinct. Even if river flooding saturated ground and raised water table, Aviva excludes indirect loss in any event. Policy definition clearly excludes rising groundwater. Flood Re cession is a premium-capping mechanism, not a coverage expansion. FOS sympathetic but cannot override clear policy wording.</t>
+        </is>
+      </c>
+      <c r="S38" s="3" t="inlineStr">
+        <is>
+          <t>Policy flood definitions using 'such as rivers, lakes and the sea' describe above-ground surface water sources that overflow — they do not include naturally occurring subsoil groundwater that rises through soil pressure. This is a physical distinction: surface overflow = flood; rising water table = groundwater (excluded). Contrast with FLOOD-035 (DRN-4415847) where same 'such as' language covered above-ground canopy water — because canopy water is above-ground overflow, not subsoil. Flood Re is a premium-risk transfer mechanism; it does not alter peril coverage.</t>
+        </is>
+      </c>
+      <c r="T38" s="3" t="inlineStr">
+        <is>
+          <t>IF cause_is_rising_water_table AND flood_definition_requires_overflow_of_external_water_sources THEN claim_excluded — water_table_is_subsoil_not_surface_overflow; IF river_flooding_raises_water_table AND policy_excludes_indirect_loss THEN groundwater_damage_excluded; flood_re_cession_does_not_expand_peril_coverage; distinguish_above_ground_external_overflow_COVERED_from_subsoil_groundwater_EXCLUDED</t>
+        </is>
+      </c>
+      <c r="U38" s="2" t="inlineStr">
+        <is>
+          <t>DRN-4948332.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="120" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-039</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5057225</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Dec 2024</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Residential buildings insurance — July 2021 basement flat flood accepted and repaired by RSA; secondary flooding appeared August 2022 on walls not replastered during original repair; RSA attributed secondary damp to pre-existing condition; policyholders argue RSA failed to complete effective and lasting repair</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>External flood — basement flat July 2021 (flood source not specified; accepted claim); secondary flooding from trapped flood water percolating through walls behind waterproof render</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Residential (basement flat)</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>RSA denied responsibility for secondary damp/flooding, asserting it was pre-existing condition evidenced by historic injection holes to external walls; RSA claimed property dried to pre-loss moisture levels</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>RSA: historic injection holes = prior damp; moisture readings reduced from 100% to 20-40% = pre-loss baseline. Mr and Mrs B: no damp in 10 years; only walls not replastered show secondary flooding; replastered walls dry; walls still wet when painter applied second coat. FOS: no evidence property was damp at 20-40% pre-loss; injection holes alone insufficient; email chain confirmed trapped flood water percolating behind waterproof render during repair works; replastered vs non-replastered correlation confirms inadequate repair.</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>RSA to undertake repair works to all walls affected by secondary flooding to achieve effective and lasting repair; RSA to pay £350 D&amp;I compensation</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="n">
+        <v>350</v>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P39" s="5" t="inlineStr">
+        <is>
+          <t>When insurer opts to settle flood claim by way of repair, it is responsible for ensuring an effective and lasting repair is completed; pre-loss damp assertion requires evidential baseline not assumption from structural features; trapped flood water percolating through structure during repair works = insurer's liability to remediate</t>
+        </is>
+      </c>
+      <c r="Q39" s="5" t="inlineStr">
+        <is>
+          <t>Pre-loss moisture readings or surveys establishing baseline damp levels; expert report attributing secondary flooding to causes unrelated to the original flood (RSA had none)</t>
+        </is>
+      </c>
+      <c r="R39" s="5" t="inlineStr">
+        <is>
+          <t>RSA left property at 20-40% moisture — considerably high — with no evidence this matched pre-loss levels. Internal emails during repair confirmed trapped flood water percolating behind waterproof render (surveyor: not rising damp, it is trapped flood water from capillary action). Timing of secondary flooding immediately after works completed points to causal link. Correlation between replastered walls (dry) and non-replastered walls (secondary flooding) is decisive. RSA did not discuss pre-loss damp concerns or alternatives with Mr and Mrs B before proceeding with repair it knew might fail. Injection holes establish possibility of prior damp, not actuality or extent.</t>
+        </is>
+      </c>
+      <c r="S39" s="5" t="inlineStr">
+        <is>
+          <t>Insurer settling flood claim by repair must complete an effective and lasting repair — if it discovers pre-loss structural concerns that may cause the repair to fail, it must discuss alternatives (e.g. cash settlement) with the policyholder rather than proceeding with a doomed repair. Pre-loss damp defence requires affirmative evidence of pre-loss moisture levels at the extent claimed, not just structural features that might indicate prior damp. Secondary flooding correlated with areas not properly stripped and replastered is attributable to inadequate flood repair.</t>
+        </is>
+      </c>
+      <c r="T39" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_settles_by_repair AND secondary_flooding_occurs_on_areas_not_fully_stripped_replastered THEN inadequate_repair_attributable_to_insurer; IF pre_loss_damp_defence AND no_pre_loss_moisture_readings THEN defence_fails; IF trapped_flood_water_identified_during_repair_works AND no_remediation THEN insurer_liable_for_subsequent_ingress; repair_obligation_requires_effective_and_lasting_outcome_not_cosmetic_completion</t>
+        </is>
+      </c>
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5057225.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="120" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-040</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5186962</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Jul 2025</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Holiday home buildings and contents insurance — September 2022 water ingress from blocked drainpipe or drainage fault; Lloyd's declined claiming damage was not from a single insured event but from continuous gradual ingress from series of floods; property unlettable since September 2022; significant reinstatement required</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>External — drainage fault; blocked drainpipe allowed rainwater to enter holiday home; source unidentified until May 2023 when neighbour's drainage fault identified and remediated</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Residential (holiday home / rental property)</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Lloyd's: damage not from a single insured event; damage caused by rainwater entering over prolonged period = continuous or gradual damage from series of floods rather than one-off event; policy requires single insured event; gradual damage exclusion also referenced; no AD cover for buildings.</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Mr and Mrs R: blocked drainpipe = single incident; unaware of ingress until flooding visible inside; took immediate steps to investigate and remediate. Lloyd's: series of water ingress events over months = not a single insured peril event; gradual damage exclusion applies. Lloyd's own surveyor confirmed property flooded: 'over Xmas 2022 and after a particularly heavy storm the property was flooded again on a much more severe scale.' FOS: flood can occur gradually (Rohan Investments); policyholders took reasonable steps to mitigate once aware; series of floods does not defeat coverage where policyholder acted reasonably.</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>Lloyd's to accept claim under flood peril; reimburse reinstatement expenditure and replaced contents at rate paid by policyholders plus 8% simple interest; cash settle outstanding works at current market rates; pay monthly rental income losses at £991 per month from February 2024 until 3 months after outstanding works settled plus 8% interest; pay £5,000 loss of rent policy benefit plus 8% interest from January 2023; pay £1,600 total D&amp;I compensation (including £450 already offered)</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>1600</v>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P40" s="3" t="inlineStr">
+        <is>
+          <t>Flood peril (undefined in policy) = buildup of water over what should be dry land (Rohan Investments Ltd v Cunningham 1998); flood can occur gradually through slow and steady buildup; gradual damage exclusion inapplicable where policyholder takes reasonable mitigation steps once aware; insurer's unfair decline makes it liable for consequential losses beyond policy limits including loss of rental income; loss of rent policy benefit (£5,000 cap) triggered from date insurer should have accepted claim</t>
+        </is>
+      </c>
+      <c r="Q40" s="3" t="inlineStr">
+        <is>
+          <t>N/A — flood causation clear from surveyor report, video evidence of water buildup, and spread of damage; policyholder mitigation steps clearly documented</t>
+        </is>
+      </c>
+      <c r="R40" s="3" t="inlineStr">
+        <is>
+          <t>Flood = buildup of water over dry land — can occur gradually (Rohan Investments 1998). Video showed water entering at a rate causing running water buildup. Surveyor confirmed flooding. Spread of damage to flooring, walls and furniture typical of flood. Whether one flood or series: policyholders took reasonable steps once aware — investigated cause, installed drying machines, arranged CCTV, stripped back sections. Source could not be identified until May 2023 despite reasonable efforts. Gradual damage exclusion cannot apply where policyholder acted reasonably. Lloyd's unfair decline means it bears consequential rental income loss from February 2024 when property would have been relet. £5,000 loss of rent benefit payable from January 2023. £1,600 D&amp;I for significant financial distress (loans, pension drawdown, personal repair work) over extended period.</t>
+        </is>
+      </c>
+      <c r="S40" s="3" t="inlineStr">
+        <is>
+          <t>Unfair flood claim decline makes insurer liable for consequential losses beyond policy benefit limits — including rental income from date property would have been relet had claim been accepted. Series of water ingress events from unidentified latent cause = single flood claim where policyholders diligently investigate and mitigate. Gradual damage exclusion requires showing policyholder failed to act reasonably — not applicable where latent cause not identifiable despite good-faith efforts. For holiday home policies with loss of rent benefits, benefit runs from date of insured event or date insurer should have accepted claim.</t>
+        </is>
+      </c>
+      <c r="T40" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_unfairly_declines_flood_claim AND property_unlettable THEN insurer_liable_for_rental_income_loss_from_date_property_would_have_been_relet; IF series_of_water_ingress_events AND policyholder_takes_reasonable_mitigation THEN gradual_damage_exclusion_does_not_apply; flood_definition_undefined_in_policy = use_Rohan_Investments_buildup_of_water_definition; loss_of_rent_benefit_triggered_from_date_insurer_should_have_accepted_claim</t>
+        </is>
+      </c>
+      <c r="U40" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5186962.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add FLOOD-041 to FLOOD-050 to Flood Case Database - Batch 5 complete
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Flood_Case_Database.xlsx
+++ b/knowledge/case-databases/Flood_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U40"/>
+  <dimension ref="A1:U50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4698,6 +4698,1056 @@
         </is>
       </c>
     </row>
+    <row r="41" ht="120" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-041</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5267073</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>The National Farmers' Union Mutual Insurance Society Limited</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Mar 2025</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Residential buildings and contents insurance — January 2024 flood accepted by NFU; dispute about whether insurer must fund comprehensive flood defences or rebuild/lift property to prevent future flooding; NFU offered £5,000 flood resilience benefit per policy terms but declined to fund rebuild or lifting as betterment</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>External flood water — January 2024 flood event; NFU accepted the flood claim; groundwater flood risk from Chalk aquifer identified in expert flood report (moderate to high 1.3% annual probability)</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>NFU: proposed repairs are effective and lasting per independent expert flood risk report (1.3% annual probability); any further payment beyond the policy £5,000 flood resilience benefit would constitute betterment; policy does not oblige insurer to fund rebuild or lifting of property</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>NFU provided independent expert flood risk report: moderate to high 1.3% annual probability of groundwater levels rising above surface level; not necessarily indicating property will flood. Policyholders argued local mismanagement (not weather) causes higher flood risk not captured by the report. No independent expert evidence submitted by policyholders to counter NFU's report. FOS found NFU's expert report persuasive in absence of rebuttal.</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld; NFU's repair settlement (including £5,000 flood resilience benefit) is effective and lasting per expert flood report; insufficient evidence that property will definitely re-flood post-repair; NFU not required to fund rebuild or lift property</t>
+        </is>
+      </c>
+      <c r="N41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P41" s="5" t="inlineStr">
+        <is>
+          <t>Flood resilience benefit clause: up to £5,000 for flood resilience measures where repair cost &gt;£10,000 with prior insurer consent; 'effective and lasting repair' principle — FOS requires evidence that repair will not be effective and lasting before ordering betterment; betterment principle limits insurer liability to like-for-like repair not structural enhancements</t>
+        </is>
+      </c>
+      <c r="Q41" s="5" t="inlineStr">
+        <is>
+          <t>Independent expert evidence on local flood risk factors (drainage/watercourse mismanagement) to counter insurer's flood risk report; expert evidence that property will definitely flood again post-repair</t>
+        </is>
+      </c>
+      <c r="R41" s="5" t="inlineStr">
+        <is>
+          <t>FOS principle: repairs must be effective and lasting. To require insurer to fund rebuild/lift, consumer must show property will definitely flood again post-repair. NFU's independent expert flood risk report (1.3% annual probability, moderate risk) was uncontested by independent expert counter-evidence. Consumer's assertion of local mismanagement as a higher-risk factor was not evidenced. Without rebuttal of insurer's expert report, FOS cannot order betterment beyond policy benefit cap.</t>
+        </is>
+      </c>
+      <c r="S41" s="5" t="inlineStr">
+        <is>
+          <t>Where flood claim is accepted and dispute concerns flood defences/betterment, insurer must obtain and rely on independent expert flood risk assessment. Consumer must provide specific expert evidence to rebut that assessment — general assertions about local conditions are insufficient. The policy flood resilience benefit is capped and conditional; further flood prevention beyond that cap requires proof of definite re-flooding risk. FOS cannot direct insurer to fund betterment on basis of possibility alone.</t>
+        </is>
+      </c>
+      <c r="T41" s="5" t="inlineStr">
+        <is>
+          <t>IF flood_claim_accepted AND dispute_about_flood_defences AND insurer_has_independent_flood_risk_report AND consumer_provides_no_expert_rebuttal THEN decline_flood_prevention_beyond_policy_benefit_cap; repair_deemed_effective_and_lasting_unless_consumer_demonstrates_definite_reflooding_risk</t>
+        </is>
+      </c>
+      <c r="U41" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5267073.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="120" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-042</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5285327</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>U K Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Feb 2025</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Residential buildings insurance — water pooling under floorboards from rising water table following heavy rainfall; Churchill declined claim as water table changes constitute neither storm nor flood; all parties agreed rising water table was the cause</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Groundwater — rising water table; water pooled under floorboards as water table increased beneath property; all three parties (Churchill's loss adjuster, Churchill's drying specialist, consumer's builder) independently agreed water table rise was cause</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Churchill: rainfall did not meet policy storm threshold; gradual water table fluctuation is not a flood (no sudden/violent event; loss adjuster definition required event such as river bursting its banks or coastal flooding); policy includes gradual damage exclusion; no sudden release of water identifiable</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>All three parties — Churchill's loss adjuster, Churchill's drying specialist, and consumer's own builder — independently agreed rising water table caused water to pool under property. No factual dispute on cause. Dispute was definitional: Churchill argued flood requires sudden/violent external event and applied extra-contractual narrow definition; policy had no flood definition. FOS: no policy flood definition exists; FOS broad definition applies; gradual water table rise causing pooling = flood.</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr">
+        <is>
+          <t>Complaint upheld; Churchill must reconsider claim under flood peril; gradual water table rise causing water to pool under property constitutes flood where policy has no flood definition; Churchill must then assess whether the flood caused the specific damage claimed (damage to solom/damp proof course)</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P42" s="3" t="inlineStr">
+        <is>
+          <t>Flood peril (undefined in policy) — where no flood definition exists FOS applies broad definition: flood can occur gradually through slow and steady build-up of water including rising water table; insurer cannot apply extra-contractual narrow flood definition (rivers/coastal only) not set out in policy terms; all-party consensus on cause of water entry is decisive on flood peril question</t>
+        </is>
+      </c>
+      <c r="Q42" s="3" t="inlineStr">
+        <is>
+          <t>Evidence of whether the flood (water table rise) specifically caused the claimed damage to the solom/damp proof course — Churchill had not assessed this when declining</t>
+        </is>
+      </c>
+      <c r="R42" s="3" t="inlineStr">
+        <is>
+          <t>All parties agreed water table rise caused water to pool under property — no factual dispute. Churchill's policy has no flood definition. Churchill cannot apply an extra-contractual narrow definition requiring sudden/violent event or specific external source (rivers, coastal) when that definition is not in the policy. FOS broad definition: flood can occur gradually through slow and steady water build-up; water table rise causing pooling = flood. Churchill must now assess whether the flood caused the specific claimed damage.</t>
+        </is>
+      </c>
+      <c r="S42" s="3" t="inlineStr">
+        <is>
+          <t>If policy has no flood definition and insurer declines on grounds water table rise is not a flood, FOS will apply its broad flood definition and require reconsideration. Loss adjuster conceding water table rise as cause while arguing it is not a flood is inconsistent where no policy definition supports that distinction. All-party agreement on cause of water entry is decisive on flood peril question. Reconsideration does not automatically mean payment — insurer must still assess causation of specific damage.</t>
+        </is>
+      </c>
+      <c r="T42" s="3" t="inlineStr">
+        <is>
+          <t>IF policy_has_no_flood_definition AND water_table_rise_causes_water_to_pool_under_property AND all_parties_agree_on_cause THEN classify_as_flood_and_reconsider; IF insurer_applies_extra_contractual_narrow_flood_definition THEN FOS_overrides_with_broad_definition; gradual_water_table_rise_can_constitute_flood_where_water_enters_or_pools_in_property</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5285327.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="120" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-043</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5349922</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Covea Insurance plc</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Mar 2025</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Flood insurance premium repricing dispute — no flood claim; Covea increased buildings and contents premium from £3,521 to £5,220 at March 2024 renewal citing increased flood risk assessment; Covea also sent renewal documents late (after renewal date), denying consumer opportunity to shop around</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no flood occurred; dispute concerns flood risk assessment methodology used for underwriting and late communication of renewal premium</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>Claim Recording / Administrative Dispute</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>N/A — no claim made; Covea's premium increase driven by Flood Zone 2 classification within 25m boundary radius per proprietary risk algorithm exceeding Covea's underwriting threshold, triggering Flood Re referral and removal of discounts</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>Covea: proprietary risk data shows Flood Zone 2 within 25m boundary; algorithm produces overall flood score above underwriting threshold; data applied consistently to all customers. Consumer: Environment Agency data shows 'Very Low' flood risk (&lt;0.1%); property built 1m higher than neighbours; never flooded in 41 years; 25m radius methodology arbitrary. FOS: FOS cannot override insurer's consistent proprietary pricing methodology; government data is one input among many; Covea acted consistently and without discrimination.</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>Premium pricing upheld as fair and consistently applied; £200 compensation awarded for late renewal documents (not received until 8 days after renewal date), which denied consumer opportunity to compare alternatives before cover auto-renewed at significantly increased premium</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P43" s="5" t="inlineStr">
+        <is>
+          <t>FCA ICOBS consumer fairness principles — insurer must provide timely renewal documents to allow consumer to make informed decision before renewal; FOS cannot direct insurer on premium pricing methodology if applied consistently to all customers in same risk profile without discrimination or data error; Flood Re referral is risk transfer mechanism not a coverage change; insurer's flood risk assessment can consider area within defined radius of property boundary</t>
+        </is>
+      </c>
+      <c r="Q43" s="5" t="inlineStr">
+        <is>
+          <t>N/A — pricing methodology dispute; FOS cannot compel use of alternative risk data source</t>
+        </is>
+      </c>
+      <c r="R43" s="5" t="inlineStr">
+        <is>
+          <t>FOS has no power to override insurer's pricing methodology where applied consistently to all customers and no discrimination or data error demonstrated. Covea's 25m boundary radius methodology applied uniformly; their data legitimately showed Flood Zone 2 proximity. Not a data error. However, renewal documents not sent until 8 days after renewal date — consumer missed ability to shop around before policy auto-renewed at higher premium. Cover had already started when documents arrived. £200 compensation reflects loss of opportunity to compare alternatives at significant premium uplift.</t>
+        </is>
+      </c>
+      <c r="S43" s="5" t="inlineStr">
+        <is>
+          <t>FOS cannot interfere with insurer's flood risk underwriting methodology if applied consistently without data error — consumers cannot compel insurers to price risk using government data over proprietary models. However, late renewal documentation for significant premium increases is a separate administrative failure: consumer must have timely pre-renewal notice to exercise right to shop around. Flood Re referral means insurer can no longer offer discounts on the flood element of the premium.</t>
+        </is>
+      </c>
+      <c r="T43" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_applies_consistent_proprietary_flood_risk_methodology AND no_discrimination_or_data_error THEN premium_challenge_fails; IF renewal_documents_sent_after_renewal_date AND premium_significantly_increased THEN compensation_for_loss_of_ability_to_shop_around; FOS_cannot_direct_insurer_to_use_alternative_flood_risk_data_source</t>
+        </is>
+      </c>
+      <c r="U43" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5349922.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="120" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-044</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5387216</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Covea Insurance plc</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Apr 2025</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Residential buildings and contents insurance — March 2024 cellar flood from rising water table through cracks in walls and floor; Covea accepted some damage but declined flood prevention measures (tanking, larger sump pump) as betterment; Covea characterised flood as one-off; property flooded again in early 2025</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Groundwater — temporary rise in water table caused water ingress through cracks in cellar walls and floor; sump pump insufficient to manage ingress; Covea's own expert acknowledged no guarantee standard repairs would be sufficient under high water pressure</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Residential home (with cellar/basement)</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Covea: cracks in cellar walls and floor were due to long-standing wear and tear/deterioration; flood was a one-off incident with no foreseeable risk of recurrence; flood prevention measures (tanking) constitute betterment as consumer did not have tanking previously; government flood risk data showed no significant flood risk</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>Covea's expert: water entered from 3 areas — repairs possible but 'no guarantee measures will be sufficient should water pressures be overbearing'; 'as basement is not tanked, it is anticipated there will be some moisture/dampness; should water table have risen, further works likely necessary'. Property flooded again in early 2025 in similar manner. FOS: Covea's own expert report undermined the 'one-off' characterisation; consecutive years of flooding disproves it definitively.</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>Complaint upheld; Covea must arrange and pay for suitable flood prevention measures (agreed between parties with their experts) to make the repair effective and lasting; betterment argument overridden by consecutive floods in 2024 and 2025 and Covea's own expert acknowledgement of ongoing risk; £250 D&amp;I compensation</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P44" s="3" t="inlineStr">
+        <is>
+          <t>'Effective and lasting repair' principle — where property at significant risk of re-flooding, flood prevention measures are required to make repair effective and lasting rather than a repair that will need redoing after a short period; betterment argument fails where insurer's own expert acknowledges repair may be insufficient under certain conditions AND property subsequently re-floods; betterment principle cannot prevent insurer from funding measures necessary for durable repair</t>
+        </is>
+      </c>
+      <c r="Q44" s="3" t="inlineStr">
+        <is>
+          <t>Covea's final response contradicted by own expert report which qualified repair effectiveness; second flood in 2025 provided conclusive real-world evidence against one-off characterisation</t>
+        </is>
+      </c>
+      <c r="R44" s="3" t="inlineStr">
+        <is>
+          <t>Covea's final response claimed one-off event with no foreseeable recurrence risk — directly contradicted by Covea's own expert who acknowledged 'no guarantee' of sufficiency under high water pressure and anticipated further works if water table risen. Property then flooded again in early 2025 in same manner, definitively disproving one-off characterisation. FOS principle: repairs must be effective and lasting; no point completing repair work requiring redoing after short period. With floods in 2024 and 2025, flood prevention measures are logically necessary. Betterment argument cannot override effective-and-lasting repair obligation.</t>
+        </is>
+      </c>
+      <c r="S44" s="3" t="inlineStr">
+        <is>
+          <t>When insurer's own expert qualifies effectiveness of proposed repair AND property subsequently re-floods, betterment argument against flood prevention measures fails. The 'effective and lasting repair' principle requires insurer to fund prevention measures if short-term repair would need to be redone. A second flood within 12 months is decisive evidence against the 'one-off' defence. Where parties cannot agree on specific works, FOS can order parties to agree with their experts rather than specifying exact measures in the decision.</t>
+        </is>
+      </c>
+      <c r="T44" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_own_expert_qualifies_repair_sufficiency AND property_re_floods_within_12_months THEN flood_prevention_measures_required_for_effective_lasting_repair; IF betterment_argument AND prevention_measures_necessary_for_durability THEN betterment_argument_fails; IF cellar_or_basement AND repeated_water_table_flooding THEN tanking_or_equivalent_prevention_likely_required</t>
+        </is>
+      </c>
+      <c r="U44" s="2" t="inlineStr">
+        <is>
+          <t>DRN-5387216.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="120" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-045</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5601561</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Advantage Insurance Company Limited</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Residential home insurance — April 2024 heavy water ingress into bedroom floor of extension; consumer claimed groundwater hydrostatic pressure surge (flood); Advantage declined — consumer's own damp proofing expert (sole inspector) found structural movement evidence; Advantage's engineer confirmed hydrostatic pressure insufficient to cause observed concrete failure</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Claimed — hydrostatic pressure from groundwater surge causing damp proof membrane failure in concrete extension floor; insurer attributed damage to structural movement (differential settlement of concrete slab, possibly tree root action or poor compaction) damaging damp proof membrane; consumer's own inspector found structural movement evidence</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>Advantage: structural movement (differential settlement of concrete slab) damaged damp proof membrane — not flood; structural movement is gradual cause excluded by policy; policy defines flood as external water entering at/below ground level with substantial/abnormal volume — excludes gradual seepage; consumer's own inspector (only party to physically inspect) found structural movement evidence; Advantage's senior engineer concluded hydrostatic pressure insufficient to cause observed concrete failure pattern</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>Consumer's damp proofing company (Company W, only party to physically inspect): visible structural movement caused cracks in slab and created vulnerable floor/wall junction; concluded damage caused by movement in structure which had damaged damp proof membrane. Advantage's senior engineer: concrete requires 3,500–5,000 psi of compressive strength before failure; volume of water needed would have caused far greater damage than occurred; most likely cause was differential settlement from tree root action or poor compaction. Consumer provided Met Office above-average rainfall data and Environment Agency article on groundwater flooding occurring weeks/months after rainfall. FOS: consumer's own inspector evidence and Advantage's technical analysis together favoured structural cause on balance of probabilities.</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld; consumer failed to demonstrate on balance of probabilities that flood caused the damage; structural movement (differential slab settlement) is the more likely cause per consumer's own inspector findings and Advantage's technical evidence on concrete failure thresholds; Advantage acted reasonably in declining</t>
+        </is>
+      </c>
+      <c r="N45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P45" s="5" t="inlineStr">
+        <is>
+          <t>Policyholder bears burden of proving insured event caused damage on balance of probabilities; policy flood definition: water from external source entering at or below ground level with substantial and abnormal volume/weight/force; excludes gradual seepage/rising damp; where consumer's own expert evidence supports alternative (non-flood) structural cause, claim properly declined; consumer's refusal of further investigation under alternative perils means insurer need not take further action</t>
+        </is>
+      </c>
+      <c r="Q45" s="5" t="inlineStr">
+        <is>
+          <t>Independent structural engineer report contradicting consumer's own inspector's structural movement conclusion; consumer declined Advantage's offer to investigate further under alternative perils (e.g. subsidence); hydrostatic pressure measurements at time of event</t>
+        </is>
+      </c>
+      <c r="R45" s="5" t="inlineStr">
+        <is>
+          <t>Consumer's own damp proofing company (only party to physically inspect property) found structural movement in concrete slab — cracks, vulnerable floor/wall junction — and concluded damp proof membrane was damaged by structural movement. Advantage's senior engineer provided technical reasoning why hydrostatic pressure from groundwater would be insufficient to cause observed concrete failure (failure thresholds require volumes that would have caused far greater damage). Consumer's Met Office and EA evidence establishes heavy rainfall and groundwater possibility but not that hydrostatic pressure specifically caused this failure pattern. Balance of probabilities favours structural movement. Consumer also declined Advantage's offer of further investigation under alternative perils.</t>
+        </is>
+      </c>
+      <c r="S45" s="5" t="inlineStr">
+        <is>
+          <t>Where consumer's own expert (sole inspector) concludes structural movement caused damage, insurer's decline on that basis is appropriate even if consumer disputes that finding. Consumer cannot selectively cite inspector's positive observations (rainfall/groundwater) while ignoring inspector's structural movement conclusion. Consumer refusal of further investigation under alternative perils (subsidence) weakens their position and means insurer need not act further. Technical evidence on concrete failure thresholds (psi requirements) is persuasive in defeating hydrostatic pressure flood theory.</t>
+        </is>
+      </c>
+      <c r="T45" s="5" t="inlineStr">
+        <is>
+          <t>IF consumers_own_inspector_finds_structural_movement_evidence AND insurer_provides_technical_evidence_hydrostatic_pressure_insufficient_to_cause_damage_pattern THEN decline_on_balance_of_probabilities; IF consumer_declines_further_investigation_under_alternative_perils THEN insurer_need_not_take_further_action; concrete_failure_threshold_evidence_defeats_hydrostatic_pressure_flood_theory</t>
+        </is>
+      </c>
+      <c r="U45" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5601561.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="120" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-046</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>DRN5640983</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Jun 2020</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Residential home insurance — water damage to converted basement through failed tanking; RSA declined claiming damage attributable to wear and tear or gradual causes; RSA acknowledged it had not had sufficient time to investigate flood as a potential cause before declining</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>Water ingress through failed tanking in converted basement; RSA attributed to wear and tear or gradual causes; water table rise identified as possible alternative cause but RSA claimed specifically excluded by policy; precise flood source not established before claim was declined</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Residential home (with converted basement)</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>RSA: no insured peril occurred; damage attributable to wear and tear or gradual cause (tanking failure); flood requires sudden/violent event or established external cause (RSA's loss adjuster position); water table rise is specifically excluded by policy; RSA acknowledged it had insufficient time to investigate flood cause before declining</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>RSA obtained loss adjuster report and drains survey — no pipe/drain issues found; attributed damage to tanking failure and lack of DPM (wear and tear). Consumer obtained report that basement needed tanking protection from groundwater; paid for rectification including tanking and waterproofing. FOS investigator: flood can occur gradually through slow and steady build-up (court-established principle); RSA failed to eliminate flood as cause before declining. RSA response: courts require established clear external cause for flood; water table is specifically excluded; investigator's broad definition is flawed. RSA acknowledged insufficient investigation time — FOS: must reassess.</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>Complaint upheld; RSA must reassess claim against flood peril using FOS broad flood definition (water building up slowly and steadily in a property can constitute flood regardless of source); RSA not yet required to pay claim — must first obtain expert evidence on flood as cause then respond accordingly</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P46" s="3" t="inlineStr">
+        <is>
+          <t>Flood peril (undefined in policy) — FOS broad definition: flood can occur when water enters or builds up in a property slowly and steadily regardless of source; insurer cannot decline for wear and tear/gradual without first completing investigation to eliminate flood as a potential cause; burden of proving exclusion applies rests with insurer; insurer's acknowledgement of incomplete investigation is significant</t>
+        </is>
+      </c>
+      <c r="Q46" s="3" t="inlineStr">
+        <is>
+          <t>RSA acknowledged it did not complete investigation of flood as potential cause before declining; expert evidence on whether accumulated water in basement constituted flood under FOS broad definition</t>
+        </is>
+      </c>
+      <c r="R46" s="3" t="inlineStr">
+        <is>
+          <t>RSA declined without completing investigation to eliminate flood as potential cause — and acknowledged this. FOS approach: flood can occur gradually through slow and steady water build-up. Key question: was water building up in basement in a way that constitutes flood? RSA has not properly investigated this. RSA must reassess against flood peril (not necessarily pay at this stage) — obtain expert evidence on cause, then respond. If further dispute arises, consumers can bring new complaint.</t>
+        </is>
+      </c>
+      <c r="S46" s="3" t="inlineStr">
+        <is>
+          <t>Insurer cannot decline basement/cellar water damage for wear and tear without first properly investigating and eliminating flood as a cause. FOS applies broad flood definition to basement water ingress: slow water build-up qualifies as flood regardless of source. Acknowledgement by insurer of incomplete investigation is dispositive — cannot maintain decline without completing investigation. Correct process: investigate → obtain expert evidence → then decide. Reassessment order does not necessarily result in payment.</t>
+        </is>
+      </c>
+      <c r="T46" s="3" t="inlineStr">
+        <is>
+          <t>IF insurer_declines_basement_water_damage AND insurer_acknowledges_incomplete_flood_investigation THEN FOS_orders_reassessment; IF no_policy_flood_definition AND water_builds_up_slowly_in_basement THEN apply_broad_FOS_flood_definition; insurer_must_eliminate_flood_as_cause_before_relying_on_wear_and_tear_exclusion</t>
+        </is>
+      </c>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
+          <t>DRN5640983.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="120" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-047</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5827621</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Aviva Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Sep 2025</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Residential buildings and contents insurance — October 2023 flood accepted by Aviva; dispute about scope of flood damage coverage (kitchen, downstairs bathroom not fully covered); Aviva's contractor fitted cloakroom joists not to building regulations; Aviva's delay in upstairs drying caused consequential bedroom mould</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>External flood water — October 2023 flood event (source not specified); Aviva accepted flood entered property and damaged hallway and part of kitchen flooring; dispute about whether flood water reached full kitchen, bathroom, and whether contractor caused further damage</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>Aviva: moisture readings taken promptly showed flood water only entered first three rows of kitchen flooring; no evidence flood reached bathroom; kitchen appliances not in kitchen at time of flood (renovation in progress); contractor repairs to cloakroom joists were appropriate; upstairs bedroom damp attributed to pre-existing damp (estate agent photos)</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>Aviva: contemporaneous moisture readings limited flood extent to kitchen flooring; estate agent photos from pre-purchase showed bedroom damp. Consumer: surveyor report (2 months later, restricted bathroom access) said all ground floor rooms affected; moisture readings unreliable; contractor damaged waste pipe and fitted joists not to building regulations; all damp caused by flood and Aviva's drying delay. FOS: contemporaneous moisture readings outweigh later surveyor report with restricted access; contractor's detailed expert report proved non-compliant joist fitting; drying delay caused avoidable upstairs mould.</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>Aviva must pay: £200 toward cloakroom joist replacement; £100 for joist inspection report (on evidence of payment); cost of fungi wash and emulsion to upstairs bedroom walls and ceilings; £150 D&amp;I compensation. Kitchen/bathroom additional claims not required.</t>
+        </is>
+      </c>
+      <c r="N47" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P47" s="5" t="inlineStr">
+        <is>
+          <t>Insurer liable for consequential damage caused by its contractor's substandard work (joist fitting not to building regulations); insurer's duty to take reasonable steps to dry property promptly after flood to prevent consequential mould; contemporaneous moisture readings from insurer outweigh later surveyor reports with restricted access; pre-existing damp documented in pre-purchase photographs limits insurer's liability for all subsequent bedroom damp</t>
+        </is>
+      </c>
+      <c r="Q47" s="5" t="inlineStr">
+        <is>
+          <t>Consumer had no contemporaneous photographs of kitchen appliances in kitchen at time of flood (photo taken 5 days later); surveyor's bathroom inspection was restricted by stored items and taken 2 months after flood</t>
+        </is>
+      </c>
+      <c r="R47" s="5" t="inlineStr">
+        <is>
+          <t>Kitchen/bathroom: contemporaneous moisture readings (taken promptly) are more reliable than surveyor report taken 2 months later with restricted bathroom inspection. Pre-existing damp in estate agent photographs limits full insurer liability for bedroom damp. Cloakroom joists: consumer's detailed contractor report with photographs proved joists did not meet building regulations — Aviva could not contest this; £200 for remediation plus £100 for report cost (if evidenced). Bedroom mould: Aviva's delay in installing upstairs drying caused avoidable mould — cost of fungi wash and emulsion awarded. £150 D&amp;I for drying delay and non-compliant joist discovery.</t>
+        </is>
+      </c>
+      <c r="S47" s="5" t="inlineStr">
+        <is>
+          <t>Insurer's contemporaneous moisture readings taken promptly after flood are the most reliable evidence of flood extent; later surveys with restricted access carry less weight. Where insurer's contractor fails to meet building regulations in repair work, insurer bears cost of remediation even where consumer was also carrying out private works in the same area. Delay in installing drying equipment upstairs creates liability for consequential mould that could have been avoided — limited to treatment cost (fungi wash/emulsion), not full redecoration where pre-existing damp exists.</t>
+        </is>
+      </c>
+      <c r="T47" s="5" t="inlineStr">
+        <is>
+          <t>IF contemporaneous_insurer_moisture_readings AND later_surveyor_report_with_restricted_access THEN moisture_readings_prevail_on_flood_extent; IF contractor_repair_not_to_building_regulations AND consumer_provides_detailed_expert_report THEN insurer_liable_for_remediation_cost; IF insurer_delays_upstairs_drying AND consequential_mould_occurs THEN insurer_liable_for_mould_treatment_not_full_redecoration_where_pre_existing_damp; pre_existing_damp_in_pre_purchase_photos_limits_insurer_liability</t>
+        </is>
+      </c>
+      <c r="U47" s="4" t="inlineStr">
+        <is>
+          <t>DRN-5827621.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="120" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-048</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>DRN-6051732</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Allianz Global Corporate &amp; Specialty SE</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Commercial property insurance (charity) — November 2024 flood claim; Allianz said flood cover was accidentally included in policy schedule by broker (acting as Allianz's agent); flood cover was not intended at renewal; Allianz declined claim; charity forced to close and suffered significant losses</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>External flood — commercial charity premises November 2024; flood caused extensive damage and forced closure; flood source not specified in decision</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Commercial (charity premises)</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>Allianz: flood cover was excluded at renewal but broker accidentally included it in policy schedule; mutual intention at renewal was to exclude flood (October 2024 renewal invite explicitly stated no flood cover; prior 3 years' policies excluded flood; broker instructed to renew on same terms); erroneous schedule does not create valid flood cover</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>Charity (T): schedule clearly showed flood cover; Allianz's own Loss Adjuster confirmed flood cover; schedule is legally binding contract. Allianz: renewal invite (October 2024) explicitly stated no flood; T's broker asked to renew on same terms as prior year (no flood); S (broker acting for Allianz) made the schedule error. FOS: common intention at renewal was to exclude flood; Allianz was not satisfied T would have sought flood cover if schedule had been correct; Allianz's delay in confirming the error (November 2024 to January 2025) caused T inconvenience warranting £250 compensation.</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Compensation Only</t>
+        </is>
+      </c>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>Flood claim not required to be paid — flood cover was not genuinely in place; £250 compensation to T for inconvenience of being led to believe claim was being considered under valid flood cover while Allianz investigated and confirmed error in January 2025</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P48" s="3" t="inlineStr">
+        <is>
+          <t>Policy schedule error by broker acting as insurer's agent — mutual intention at renewal governs true policy coverage despite schedule error; FOS applies fairness standard not strict contractual enforcement; prior policy history (3 years without flood cover) and renewal documentation (explicit flood exclusion) are evidence of mutual intention; delay in communicating coverage error causes inconvenience warranting D&amp;I compensation even where underlying claim fails</t>
+        </is>
+      </c>
+      <c r="Q48" s="3" t="inlineStr">
+        <is>
+          <t>N/A — mutual intention clear from renewal invite, prior 3 years' policies, and broker's instruction to renew on same terms; no evidence T would have sought alternative flood cover</t>
+        </is>
+      </c>
+      <c r="R48" s="3" t="inlineStr">
+        <is>
+          <t>FOS is not a contract enforcement body. On fairness: mutual intention at renewal was clearly to exclude flood (renewal invite said so; broker asked to renew on same terms; 3 prior years had no flood cover). Erroneous schedule did not reflect what was agreed. Allianz taking from November 2024 to January 2025 to identify and confirm the error meant T was led to believe claim was being considered — T could not take alternative action in that period. £250 compensation for that inconvenience. No additional material loss causally established from the period of erroneous claim consideration.</t>
+        </is>
+      </c>
+      <c r="S48" s="3" t="inlineStr">
+        <is>
+          <t>Where insurer's broker accidentally includes cover in schedule that was explicitly excluded in renewal documents, FOS looks to mutual intention (renewal terms agreed, prior policy history) rather than schedule to determine actual coverage. Insurer's time in identifying and communicating schedule error causes inconvenience even where no material loss results — warrants modest D&amp;I compensation. Evidence of mutual intention: prior policy history without that cover, broker's renewal instruction on same terms, and renewal documentation pre-dating the erroneous schedule.</t>
+        </is>
+      </c>
+      <c r="T48" s="3" t="inlineStr">
+        <is>
+          <t>IF policy_schedule_includes_cover AND renewal_documents_explicitly_excluded_cover AND broker_asked_to_renew_on_same_terms AND prior_policies_excluded_cover THEN erroneous_schedule_does_not_create_valid_cover; IF insurer_delays_confirming_schedule_error AND claimant_led_to_believe_claim_being_considered THEN D_and_I_compensation_warranted; mutual_intention_at_renewal_governs_coverage_despite_schedule_errors</t>
+        </is>
+      </c>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
+          <t>DRN-6051732.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="120" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-049</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>DRN6137899</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>UK General Insurance (Ireland) Limited</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>May 2015</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Commercial shop insurance (public liability and business interruption) — sewer surge from water company caused flooding at shop (fourth flood at premises); dispute about floor replacement under public liability (insurer cannot produce policy copy), business interruption payment (insufficient evidence provided), and recovery of uninsured losses from water company</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Sewer surge — water company's responsibility; surged sewer caused flooding at commercial shop premises; fourth flood at the same premises from same cause</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>Commercial (shop/business premises)</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>UKI: floor claim rejected under public liability — expert evidence suggested floor damage occurred over long period from previous floods (pre-policy inception); business interruption declined pending consumer providing daily trading statements (annual accounts insufficient); uninsured loss recovery from water company: UKI eventually withdrew assistance when consumer could not provide required evidence before limitation period</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>UKI: cannot produce full policy copy (only business interruption section); floor damage pre-dates policy inception per expert evidence; Mr and Mrs P did not provide daily trading statements for BI claim. Consumer: shop closed longer than UKI thinks; supplied annual accounts (not daily statements); UKI confused responsibility for water company recovery; Mrs P's serious illness prevented responding to UKI's requests. FOS: without policy copy UKI cannot apply exclusions; public liability trigger is when liability to landlord arose (post-inception), not when damage occurred; BI claim requires specific daily trading statements not annual accounts.</t>
+        </is>
+      </c>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M49" s="5" t="inlineStr">
+        <is>
+          <t>UKI must reconsider floor claim under public liability without applying exclusions (cannot evidence exclusions without policy copy); UKI must reconsider business interruption claim if consumer provides daily trading statements for closure period within covered period; uninsured loss recovery handling upheld as reasonable voluntary assistance; no D&amp;I compensation awarded</t>
+        </is>
+      </c>
+      <c r="N49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" s="4" t="inlineStr">
+        <is>
+          <t>No — Commercial</t>
+        </is>
+      </c>
+      <c r="P49" s="5" t="inlineStr">
+        <is>
+          <t>Insurer who cannot produce relevant policy sections cannot apply exclusions in those sections — burden of proving exclusion rests with insurer; public liability trigger is when liability to third party (landlord) arose, not when physical damage occurred (relevant for cumulative/historical damage); business interruption requires policyholder to provide evidence of losses within coverage period (daily trading statements not annual accounts); insurer's voluntary assistance with uninsured loss recovery from third party creates no ongoing obligation</t>
+        </is>
+      </c>
+      <c r="Q49" s="5" t="inlineStr">
+        <is>
+          <t>Full policy document (public liability section not available); daily trading statements for business interruption claim (only annual accounts provided)</t>
+        </is>
+      </c>
+      <c r="R49" s="5" t="inlineStr">
+        <is>
+          <t>Without policy copy, UKI cannot show what exclusions or limitations applied to public liability floor claim. Public liability trigger is when liability to landlord arose (post-inception) not when floor was originally damaged — historical damage argument therefore uncertain without seeing policy terms. UKI must reconsider floor claim without applying unproven exclusions. Business interruption: shop closed only 1.5 days within covered period; consumer must provide daily trading statements (not annual accounts) to quantify losses. Water company recovery: UKI maintained active pursuit for 4+ years and contacted parties monthly; withdrew only when evidence not forthcoming and limitation period approaching — reasonable decision not attributable to UKI's fault.</t>
+        </is>
+      </c>
+      <c r="S49" s="5" t="inlineStr">
+        <is>
+          <t>Insurer who cannot produce policy document cannot apply its exclusions — burden of proving exclusion rests with insurer who must evidence the terms they seek to rely on. Public liability cover triggers when liability arises (post-inception), not when physical damage accumulated — relevant for latent or cumulative flood damage to third-party property. Voluntary assistance with third-party recovery creates no obligation — insurer can withdraw when evidence is not forthcoming without incurring liability. Consumer must provide appropriate evidence type for BI claims: daily/weekly trading statements, not annual accounts.</t>
+        </is>
+      </c>
+      <c r="T49" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_cannot_produce_policy_document THEN insurer_cannot_apply_exclusions; IF public_liability_cover AND physical_damage_pre_inception AND liability_to_third_party_arose_post_inception THEN claim_potentially_valid; IF insurer_voluntarily_pursues_third_party_recovery AND evidence_not_forthcoming AND limitation_approaching THEN insurer_can_withdraw_without_liability; BI_claim_requires_daily_or_weekly_trading_statements_not_annual_accounts</t>
+        </is>
+      </c>
+      <c r="U49" s="4" t="inlineStr">
+        <is>
+          <t>DRN6137899.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="120" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-050</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>DRN6619758</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>International Insurance Company of Hannover SE</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Jan 2018</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Residential home insurance — water damage and mould under carpet from moisture ingress into floor void through low-set air bricks; consumer claimed flood (external water ingress); insurer declined — five independent experts all agreed cause was rot from water ingress through air bricks and poor ventilation, with no evidence of standing water accumulating in void</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Water ingress through low-set air bricks into floor void; external ground level too high relative to air bricks allowing rain water to seep into void; poor ventilation in void caused retained moisture and rot — no evidence of standing water accumulation; cause was wet ground conditions not flood</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>IICH: damage caused by rot and gradual processes (both excluded by policy); no flood demonstrated — five experts agreed water entered void through air bricks causing rot from poor ventilation and moisture; no evidence of water building up and remaining as standing water on top of ground; consumer failed to discharge burden of proving flood occurred</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>Five independent experts all agreed: cause was rot in flooring from water ingress through air bricks and inadequate ventilation; no standing water in void; external ground level too high relative to air bricks. Consumer: external water ingress = flood; consensus on external water source satisfies flood definition; no standing water because ground was soil (absorbed it). FOS: water ingress that soaks into soil without accumulating as standing water = wet ground, not flood; flood requires water to build up on top of ground; consumer failed to prove flood occurred.</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M50" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld; consumer failed to demonstrate that a flood occurred; water ingress that soaks into soil without accumulating as standing water is not a flood; all five experts agreed cause was rot from gradual moisture ingress and poor ventilation, not a flood event; IICH acted fairly in declining</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P50" s="3" t="inlineStr">
+        <is>
+          <t>Flood requires standing water to accumulate on top of ground — mere water ingress or seepage that soaks into soil without accumulating as standing water is not a flood ('wet ground' is not flood); policyholder bears burden of proving insured event caused damage on balance of probabilities; gradual damage exclusion and rot exclusion are secondary — only relevant once consumer first proves an insured event occurred; five-expert consensus on non-flood cause is decisive</t>
+        </is>
+      </c>
+      <c r="Q50" s="3" t="inlineStr">
+        <is>
+          <t>Evidence of standing water accumulating in floor void (all experts found none — ground was soil that absorbed water); evidence of a specific identifiable flood event (as opposed to general water ingress over time)</t>
+        </is>
+      </c>
+      <c r="R50" s="3" t="inlineStr">
+        <is>
+          <t>FOS definition of flood requires water to build up and sit on top of ground as standing water — not merely for water to soak into soil leaving it damp. Consumer's own argument (no standing water because soil absorbed it) proves absence of flood: water soaking into soil without accumulating is just wet ground. Five independent experts agreed water entered through air bricks, soil became damp, rot resulted from moisture and poor ventilation — no evidence of standing water accumulation. Consumer failed to discharge burden of proving flood occurred on balance of probabilities. Exclusions for gradual damage and rot are secondary — only become relevant after insured event is first established.</t>
+        </is>
+      </c>
+      <c r="S50" s="3" t="inlineStr">
+        <is>
+          <t>Flood requires standing water to accumulate on top of ground — not just water ingress that soaks into soil. Where multiple independent experts agree cause was rot/moisture/poor ventilation (not flood) and no evidence of standing water accumulation exists, claim properly declined. Gradual damage and rot exclusions are secondary to the burden-of-proof question — they only become relevant if consumer first proves an insured event occurred. Distinguish: damp soil under floor from air brick seepage (not flood) vs water building up under floorboards or in basement as standing water (potential flood).</t>
+        </is>
+      </c>
+      <c r="T50" s="3" t="inlineStr">
+        <is>
+          <t>IF all_independent_experts_agree_cause_was_rot_from_gradual_water_ingress AND no_evidence_of_standing_water_accumulation THEN claim_fails_on_balance_of_probabilities; flood_requires_standing_water_accumulation_not_mere_soil_dampness_or_seepage; IF consumer_fails_to_prove_insured_event THEN exclusions_not_relevant; five_expert_consensus_on_non_flood_cause_is_decisive_where_no_counter_evidence</t>
+        </is>
+      </c>
+      <c r="U50" s="2" t="inlineStr">
+        <is>
+          <t>DRN6619758.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add FLOOD-051 to FLOOD-056 to Flood Case Database — Batch 6 complete (Flood database final)
</commit_message>
<xml_diff>
--- a/knowledge/case-databases/Flood_Case_Database.xlsx
+++ b/knowledge/case-databases/Flood_Case_Database.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U50"/>
+  <dimension ref="A1:U56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5748,6 +5748,636 @@
         </is>
       </c>
     </row>
+    <row r="51" ht="120" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-051</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>DRN7363961</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Lloyds Bank General Insurance Limited</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>2014 (est.)</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Home insurance — 2012 flood damage claim; insurer avoided policy from commencement (2010) for alleged non-disclosure at inception of previous flood claims (2004) and prior insurance refusals; consumer (Ms B) states she disclosed both facts to a branch representative during a 2010 in-branch meeting</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>External flood water — 2012 flood event at residential home; nature of flood source not specified; flood claim triggered discovery of alleged non-disclosure at 2010 policy inception</t>
+        </is>
+      </c>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>Coverage Dispute</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>Lloyds Bank: Ms B did not disclose previous flood claims or prior insurance refusals during the 2010 branch meeting; branch representative (a branch manager) would have been unable to provide a quotation if such facts had been disclosed; application records show no such disclosure; policy documentation sent post-inception recorded no prior flood or refusal; therefore policy validly avoided from commencement</t>
+        </is>
+      </c>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>Lloyds Bank: application records show no prior flood or refusal; branch manager had no reason to falsify records; NCD documentation reflects 6-year claims-free period as a maximal NCD band, not as evidence of 2004 flood disclosure; 2011 flood incident not disclosed at 2012 renewal. Ms B: disclosed prior 2004 flood and prior refusals to branch representative; visited branch for unrelated matter and was approached about home insurance; provides detailed account of 2010 meeting. FOS: Ms B's consistent prior practice of disclosing flood claims (confirmed by refusals from multiple insurers including Lloyds Bank itself); account of meeting credible; 6-year NCD documentation consistent with 2004 flood disclosure (disclosing a 2004 claim in 2010 = 6 years); 2011 unclaimed flood need not be disclosed at renewal in response to 'circumstances changed' question.</t>
+        </is>
+      </c>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M51" s="5" t="inlineStr">
+        <is>
+          <t>Policy must be reinstated (subject to premiums being paid) and 2012 flood claim reconsidered on its merits; records of policy voidance removed from internal and external databases; £200 D&amp;I compensation; if Mr A and Ms B paid increased premiums due to the voidance, Lloyds Bank must reimburse the amount attributable solely to the voidance with 8% simple interest from date paid to settlement</t>
+        </is>
+      </c>
+      <c r="N51" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="O51" s="4" t="inlineStr">
+        <is>
+          <t>No — Administrative</t>
+        </is>
+      </c>
+      <c r="P51" s="5" t="inlineStr">
+        <is>
+          <t>Balance of probabilities standard applies to determine what was disclosed at policy inception where no recording exists; consumer's consistent prior disclosure practice across multiple insurers is strong circumstantial evidence of disclosure to this insurer; consumer reasonably entitled to believe disclosed information was accurately recorded without verifying post-sale documentation; renewal question asking if 'circumstances had changed' does not necessarily require disclosure of a prior flood event that was not claimed for (especially where third party accepted liability)</t>
+        </is>
+      </c>
+      <c r="Q51" s="5" t="inlineStr">
+        <is>
+          <t>Recording or contemporaneous written record of the 2010 branch meeting discussion</t>
+        </is>
+      </c>
+      <c r="R51" s="5" t="inlineStr">
+        <is>
+          <t>Pattern of disclosure established: Ms B was previously refused cover due to disclosing flood claims to multiple insurers including Lloyds Bank, proving consistent disclosure practice. Her account of the 2010 meeting credible: she visited for an unrelated reason with no incentive to withhold material facts when approached about insurance. NCD documentation recording 6 years claims-free is consistent with a disclosed 2004 flood claim (exactly 6 years prior). On 2011 non-claimed flood: 'circumstances changed' renewal question does not necessarily lead a consumer to disclose an event not claimed for, particularly where the council accepted liability. Balance of probabilities favours Ms B having disclosed both material facts.</t>
+        </is>
+      </c>
+      <c r="S51" s="5" t="inlineStr">
+        <is>
+          <t>Policy voidance for non-disclosure must be proven by insurer on balance of probabilities. Circumstantial evidence of consistent prior disclosure practice can outweigh application records where no recording of the inception conversation exists. Consumer's consistent pattern of disclosing material facts to prior insurers (evidenced by refusals arising from those disclosures) is strong evidence of continued disclosure. Post-sale documentation errors do not necessarily override what was verbally disclosed at inception. Renewal 'circumstances changed' question has limited scope — it does not necessarily capture every event that occurred since inception, particularly unclaimed events where a third party accepted responsibility.</t>
+        </is>
+      </c>
+      <c r="T51" s="5" t="inlineStr">
+        <is>
+          <t>IF insurer_avoids_policy_for_non_disclosure AND consumer_has_consistent_prior_disclosure_pattern_evidenced_by_prior_refusals AND no_recording_of_inception_meeting THEN FOS_applies_balance_of_probabilities_favouring_consumer_disclosure; IF renewal_documentation_asks_if_circumstances_changed AND consumer_experienced_flood_but_did_not_claim_AND_third_party_accepted_liability THEN non_disclosure_of_that_flood_at_renewal_is_reasonable; policy_voidance_requires_insurer_to_prove_non_disclosure_on_balance_of_probabilities</t>
+        </is>
+      </c>
+      <c r="U51" s="4" t="inlineStr">
+        <is>
+          <t>DRN7363961.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="120" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-052</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>DRN7937294</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>UK General Insurance (Ireland) Limited</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Sep 2015</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Home insurance — cellar flooded with a few inches of water; insurer's surveyor confirmed flood occurred and attributed cause to temporary rise in water table from prolonged heavy rainfall; policy contained specific exclusion for 'loss or damage caused by rising water table levels'; claim declined under exclusion; consumer also complained about poor service</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Groundwater — water table rose following weeks of heavy rainfall, causing water to rise through cellar floor; water receded within days after rainfall ceased; surveyor ruled out burst pipes or above-ground water ingress; Victorian cellar without adequate damp-proof membrane made property susceptible to water table ingress</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Residential home (with cellar)</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>UKII: surveyor confirmed flooding caused by rising water table following heavy rainfall; cellar lacks adequate damp-proof membrane; policy specifically excluded 'loss or damage caused by rising water table levels'; exclusion clearly set out in policy documentation; exclusion fair and reasonable to apply</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>UKII: surveyor inspected cellar; ruled out burst pipes and above-ground ingress; water table rise confirmed as sole cause; property not flooded in 8+ years of heavy rain suggesting general water table rise. Consumer: property built into hillside (only two of four cellar walls fully underground) making water table rise unlikely; UKII used incorrect rainfall data (Met Office SE regional = 64.84mm, not UKII's 118.8mm); if water table caused it, should have stayed flooded during subsequent 95mm of rain. FOS: checked UKII rainfall data against postcode-specific records — found UKII's figures correct; water table rise can occur on hillsides and quick drainage is consistent with hillside; exclusion clear and not unusual; 8+ years without flooding during other heavy rain periods suggests water table may have generally risen.</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>Compensation Only</t>
+        </is>
+      </c>
+      <c r="M52" s="3" t="inlineStr">
+        <is>
+          <t>Flood claim decline upheld as reasonable; UKII must pay £100 compensation to Mr and Mrs S for distress and inconvenience caused by UKII's poor service (agent's slow and unclear responses; surveyor misunderstanding about who diagnosed the cause)</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P52" s="3" t="inlineStr">
+        <is>
+          <t>Explicit 'rising water table levels' exclusion is valid, clear and not unusual in home insurance policies; insurer who agrees flooding occurred can still decline under rising water table exclusion; exclusion applies to temporary water table rises from heavy rain, not only permanent rises; water table rises can occur on hillsides, not only in low-lying areas; postcode-specific Met Office rainfall data is more reliable than regional averages; exclusion may apply even where flooding has not occurred previously</t>
+        </is>
+      </c>
+      <c r="Q52" s="3" t="inlineStr">
+        <is>
+          <t>N/A — exclusion was clear in policy; rainfall data verified by FOS using postcode-specific records; surveyor confirmed sole cause</t>
+        </is>
+      </c>
+      <c r="R52" s="3" t="inlineStr">
+        <is>
+          <t>UKII's surveyor confirmed water table rise as sole cause; UKII agreed it was a flood. FOS initially (first provisional) thought exclusion unreasonable for a temporary rainfall-driven water table rise. After UKII challenged, FOS reconsidered: property hadn't flooded in 8+ years despite other heavy rain, suggesting water table may have generally risen — making the exclusion logically applicable. Consumer's postcode-specific rainfall data argument rejected after FOS independently verified UKII's figures were correct. Hillside objection rejected: water table rises can occur on hillsides and quick drainage is explained by topography. Exclusion is clearly drafted, not unusual, and fair to apply. Service failures by UKII's agent and surveyor misunderstanding warranted modest £100 D&amp;I.</t>
+        </is>
+      </c>
+      <c r="S52" s="3" t="inlineStr">
+        <is>
+          <t>A clearly drafted 'rising water table levels' exclusion is distinct from having no flood definition. Where such exclusion exists: (a) insurer can concede flood occurred and still decline under the exclusion; (b) exclusion applies to temporary weather-driven rises, not just permanent table rises; (c) consumer cannot defeat the exclusion by pointing to hillside topography or challenging rainfall data without postcode-specific evidence. Contrast with Churchill-type cases where no policy flood definition existed — here the exclusion is express. Service failures (slow responses, surveyor attribution errors) warrant modest D&amp;I even where underlying claim decline is upheld.</t>
+        </is>
+      </c>
+      <c r="T52" s="3" t="inlineStr">
+        <is>
+          <t>IF policy_has_explicit_rising_water_table_exclusion AND surveyor_confirms_rising_water_table_as_sole_cause THEN decline_justified_regardless_of_flood_definition; rising_water_table_exclusion_applies_to_temporary_rainfall_driven_rises_not_just_permanent; water_table_rise_can_occur_on_hillsides; postcode_specific_rainfall_data_required_to_challenge_insurer_rainfall_figures; distinguish_express_water_table_exclusion_from_policies_with_no_flood_definition</t>
+        </is>
+      </c>
+      <c r="U52" s="2" t="inlineStr">
+        <is>
+          <t>DRN7937294.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="120" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-053</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>DRN7939869</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Royal &amp; Sun Alliance Insurance Plc</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Jan 2017</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Home insurance — basement flat flood from rising water table following heavy rain; RSA accepted flood cover but declined payment on basis contractor's invoice showed only preventative work (drain laying); consumer disputed that invoice included actual flood damage repairs; RSA's own telephone call with contractor revealed flood had caused a 'decent sized hole' which contractor made good when laying the drain</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Groundwater — rising water table following heavy rain flooded basement flat; RSA accepted flood peril; dispute concerns whether contractor's invoice covered actual flood damage repairs or only preventative work</t>
+        </is>
+      </c>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>Residential home (basement flat)</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>Handling / Reinstatement Dispute</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>Accepted — Disputed Settlement</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>RSA: claim form and contractor's invoice showed only preventative work (drain laying) and making good damage the contractor caused while laying the drain; no flood repair work identifiable in invoice; RSA confirmed with contractor by telephone who said only preventative work was done</t>
+        </is>
+      </c>
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>RSA: contractor confirmed by phone only preventative work done and making good contractor's own damage; invoice described drain laying. Consumer: provided photographs, video evidence and contractor's further letter asserting invoice included actual flood damage repairs; flood damaged walls and floor. FOS: in the same telephone call with RSA, contractor also mentioned flood had caused 'a decent sized hole' in the corner of the room where water entered; contractor made good all damage in that area (original flood damage + contractor's damage) when laying the drain; RSA failed to probe this disclosure.</t>
+        </is>
+      </c>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>Upheld in Part</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="inlineStr">
+        <is>
+          <t>RSA must take further steps to determine the amount payable to Mr and Mrs L for flood damage — whether by assessing further photographic/video evidence they have available, speaking again to the contractor to probe the disclosed flood damage, and/or carrying out a site visit</t>
+        </is>
+      </c>
+      <c r="N53" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O53" s="4" t="inlineStr">
+        <is>
+          <t>No — Handling Dispute</t>
+        </is>
+      </c>
+      <c r="P53" s="5" t="inlineStr">
+        <is>
+          <t>Policy covers flood damage but not preventative flood work (drain laying, item removal/storage to prevent damage or enable preventative work); insurer must adequately probe all material disclosures made during investigative conversations with contractors — including disclosures made incidentally during phone calls focused on other matters; contractor making good original flood damage while completing preventative works does not eliminate insurer's liability for that flood damage</t>
+        </is>
+      </c>
+      <c r="Q53" s="5" t="inlineStr">
+        <is>
+          <t>Specific quantification of flood damage in corner of room (not separately identified in contractor's invoice); photographic/video evidence of original flood damage before contractor commenced work</t>
+        </is>
+      </c>
+      <c r="R53" s="5" t="inlineStr">
+        <is>
+          <t>RSA correctly declined preventative drain-laying costs and item removal/storage. But in the same call confirming preventative-only work, contractor mentioned flood had caused 'a decent sized hole' in the corner where water entered, and that he had made good all damage in that area when laying the drain. RSA had the opportunity to probe this disclosure in the call but did not. This confirms there was payable flood damage. Amount is likely modest (as conceded by contractor) but RSA must now quantify it. RSA was not excused from investigating this disclosure simply because repairs had already been completed.</t>
+        </is>
+      </c>
+      <c r="S53" s="5" t="inlineStr">
+        <is>
+          <t>Insurer handling investigative calls with contractors must probe all disclosures — including incidental remarks about original damage made during calls focused on other matters. Contractor's admission of original flood damage made good during preventative works is material and requires follow-up. Distinguishing flood damage repair from flood prevention in a single contractor invoice requires thorough investigation. The fact that repairs are already complete does not mean a site visit would be valueless — photographic/video evidence and further contractor conversations remain investigative options. Failure to probe a material contractor disclosure is a handling failure justifying FOS intervention.</t>
+        </is>
+      </c>
+      <c r="T53" s="5" t="inlineStr">
+        <is>
+          <t>IF contractor_confirms_preventative_work_in_phone_call AND contractor_also_mentions_original_flood_damage_made_good_in_same_call THEN insurer_must_probe_and_quantify_flood_damage_element; preventative_flood_work_not_covered_BUT_original_flood_damage_made_good_by_contractor_IS_covered; IF claim_decline_based_solely_on_invoice_description AND consumer_disputes_description THEN insurer_must_speak_to_contractor_and_probe_all_disclosures; repairs_already_completed_does_not_prevent_further_investigation</t>
+        </is>
+      </c>
+      <c r="U53" s="4" t="inlineStr">
+        <is>
+          <t>DRN7939869.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="120" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-054</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>DRN8469463</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>TBO Services Limited</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>May 2016</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Commercial property insurance — broker (TBO Services Limited) failed to disclose P's prior flood history when completing 2015/2016 renewal statement of facts; insurer (overseas regulated, not FOS member) cancelled policy from start date for non-disclosure and declined 2015 flood claim; P seeks compensation from broker for loss of insurance proceeds</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Surface water — heavy rain causing water to enter commercial premises through doors (2015 flood event); property had prior flood claim from blocked drain in road outside property</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Commercial (business premises)</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Broker Conduct Dispute</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>TBO's renewal process: at 2015 renewal TBO did not ask P about any questions except one (piece of equipment); TBO inserted 'no history of flooding' in the statement of facts using 2014 data, despite knowing P had prior flood from a blocked road drain; insurer cancelled policy from start date for non-disclosure of flood susceptibility; TBO said P answered 'no' to flood history questions in 2014 and P should have corrected the statements of fact</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>TBO: in 2014 P was only asked about weather-caused flooding, and a blocked drain flood is not weather-caused; P should have noticed the incorrect answer in the 2015 statement of facts. FOS: TBO's own 2014 statement of fact recorded 'floor flooded from blocked drain on road' — it knew of prior flood; flooding from a blocked drain during heavy rain is reasonably attributed to weather conditions; at 2015 renewal TBO only asked one question — it inserted all other answers, including 'no history of flooding', without asking P; inserting an incorrect answer without asking the client is careless; P cannot be blamed for not noticing TBO's own insertion on page four of a form. Loss adjusters for second insurer: P's director confirmed several flash floods in the area prior to 2015. TBO: cannot produce recording of 2014 conversation.</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Upheld</t>
+        </is>
+      </c>
+      <c r="M54" s="3" t="inlineStr">
+        <is>
+          <t>TBO Services Limited must jointly with P instruct a loss adjuster to assess what (if anything) the insurer would likely have paid in respect of the 2015 flood claim if the policy had not been cancelled; TBO must then compensate P by the loss adjuster's assessed sum less the 2015/2016 premium P paid; TBO must also pay the loss adjuster's fee</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>No — Broker Dispute</t>
+        </is>
+      </c>
+      <c r="P54" s="3" t="inlineStr">
+        <is>
+          <t>Broker's duty to accurately complete insurance application and renewal statements of fact; where broker inserts answers on behalf of client without asking questions, broker assumes full responsibility for the accuracy of those answers; flooding from a blocked drain during heavy rain is reasonably characterised as weather-related and relevant to a 'history of flooding' question; broker cannot rely on client not having noticed broker's own incorrect insertion; where insurer is not FOS-regulated, FOS can order broker to compensate equivalent to what the insurer would have paid</t>
+        </is>
+      </c>
+      <c r="Q54" s="3" t="inlineStr">
+        <is>
+          <t>Recording of original 2014 conversation in which P provided flood history information (TBO could not produce this)</t>
+        </is>
+      </c>
+      <c r="R54" s="3" t="inlineStr">
+        <is>
+          <t>At 2015 renewal TBO asked P only one question; TBO inserted all other answers including 'no history of flooding' from 2014 data without discussing them with P. TBO knew from its own 2014 statement of fact that P's property had flooded from a blocked road drain. Flooding from a blocked drain during heavy rain is reasonably caused by weather conditions. TBO had a duty to discuss the 'history of flooding' question with P before inserting 'no' — especially knowing of the prior flood and especially given its own staff guidance to clarify questions where clients may be confused. TBO cannot shift responsibility to P for not spotting its incorrect insertion on page four. Underlying insurer not FOS member: FOS orders TBO to compensate equivalent to likely insurer settlement.</t>
+        </is>
+      </c>
+      <c r="S54" s="3" t="inlineStr">
+        <is>
+          <t>Brokers who insert renewal answers without re-asking questions assume responsibility for accuracy — especially for material flood history questions where a prior flood claim is known. A prior flood from a blocked drain during heavy rain counts as flood history relevant to flood risk questions. Where the underlying insurer is not FOS-regulated, FOS treats the broker as the responsible party and orders compensatory payment equivalent to lost insurer proceeds. Broker's own internal standards (staff to clarify confused answers) are used against it when it fails to follow them.</t>
+        </is>
+      </c>
+      <c r="T54" s="3" t="inlineStr">
+        <is>
+          <t>IF broker_inserts_answers_in_renewal_without_asking_client AND known_prior_flood_claim_exists AND history_of_flooding_answered_no THEN broker_liable_for_resulting_non_disclosure; flood_from_blocked_road_drain_during_heavy_rain_counts_as_flood_history; IF underlying_insurer_not_FOS_member AND broker_at_fault THEN FOS_orders_broker_to_compensate_equivalent_to_insurer_settlement; broker_cannot_blame_client_for_not_spotting_brokers_own_incorrect_insertion</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>DRN8469463.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="120" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>FLOOD-055</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>DRN9152389</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>WR Berkley Insurance (Europe) Limited</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Sep 2016</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Residential buildings insurance — 2015 flood damage; standard insurance schedule listed storm, tempest and flood as covered perils; policy endorsement specifically excluded 'damage caused by flooding'; consumer argued the schedule showed they had flood cover; insurer declined under the endorsement</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>External flood (2015 flood event; source not specified in decision; property known to be in a high flood risk area at inception)</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>Residential home</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>Berkley: endorsement on policy schedule specifically excluded 'damage caused by flooding'; endorsement overrides the standard schedule peril list; consumer signed a statement of fact at inception identifying property as high flood risk; initially property was unoccupied and all three perils (storm, tempest, flood) were excluded; when property became occupied, storm and tempest were included but flood was excluded by endorsement; endorsement clearly and expressly removed flood cover</t>
+        </is>
+      </c>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>Consumer: standard schedule listed storm, tempest and flood — they believed they had flood cover under the policy. Berkley: endorsement is a key and integral part of the policy; it clearly excluded flood while retaining storm and tempest; Berkley has since updated its standard schedule to treat storm and flood as separate perils, reflecting the original intent. FOS: endorsements are integral to any insurance policy; the flood exclusion endorsement clearly and expressly removed flood cover; not unfair or unreasonable to rely on it.</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M55" s="5" t="inlineStr">
+        <is>
+          <t>Complaint not upheld; Berkley acted fairly and reasonably in declining the flood claim under the clearly expressed flood exclusion endorsement</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P55" s="5" t="inlineStr">
+        <is>
+          <t>Endorsements form a key and integral part of an insurance policy and override the standard peril list in the policy schedule; a clear flood exclusion endorsement takes precedence over 'storm, tempest and flood' wording in the body of the schedule; consumer signed statement of fact identifying high flood risk at inception — consistent with expectation that flood cover might be excluded or restricted; standard policy schedule listing 'flood' as a peril does not guarantee flood cover where that cover is removed by endorsement</t>
+        </is>
+      </c>
+      <c r="Q55" s="5" t="inlineStr">
+        <is>
+          <t>N/A — endorsement was unambiguous; consumer's statement of fact acknowledged high flood risk at inception</t>
+        </is>
+      </c>
+      <c r="R55" s="5" t="inlineStr">
+        <is>
+          <t>Consumer signed a statement of fact at inception confirming the property was in a high flood risk area. Initially the property was unoccupied and storm, tempest and flood perils were all excluded. When the property became occupied, storm and tempest were restored to the standard peril list but flood was specifically excluded by endorsement. The endorsement was an integral part of the policy, clearly drafted, and expressly excluded flood damage. Berkley's subsequent update to its standard schedule (separating storm and flood as distinct perils) confirms the original intent was always to retain storm/tempest cover while excluding flood. Relying on the endorsement to decline was not unfair or unreasonable.</t>
+        </is>
+      </c>
+      <c r="S55" s="5" t="inlineStr">
+        <is>
+          <t>Consumers should read policy endorsements as an integral part of their cover — not as ancillary documents. An endorsement expressly removing flood cover takes precedence over the standard schedule's peril list. Where property is in a known high flood risk area and consumer signed a statement of fact to that effect at inception, a flood exclusion endorsement is expected and cannot be overridden by argument that the standard schedule listed flood. Insurer subsequently updating its standard schedule to reflect its original intent reinforces that the endorsement was a deliberate coverage limitation.</t>
+        </is>
+      </c>
+      <c r="T55" s="5" t="inlineStr">
+        <is>
+          <t>IF policy_endorsement_explicitly_excludes_flood AND standard_schedule_lists_flood_as_covered_peril THEN endorsement_overrides_schedule; IF property_known_high_flood_risk_at_inception AND flood_exclusion_endorsement_present THEN endorsement_expected_and_valid; endorsement_is_integral_part_of_policy_not_optional_addendum; standard_peril_list_does_not_guarantee_cover_where_endorsement_removes_it</t>
+        </is>
+      </c>
+      <c r="U55" s="4" t="inlineStr">
+        <is>
+          <t>DRN9152389.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="120" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>FLOOD-056</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>DRN9771710</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Mar 2017</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Holiday caravan insurance — Storm Frank caused river to burst banks and flood caravan site; caravan floated 120 metres and suffered extensive damage; policy covered storm and accidental damage but specifically excluded 'all claims due to flood'; insurer declined under flood exclusion; consumer argued storm was the true (proximate) cause</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Flood water from river bursting banks — Storm Frank conditions (sustained winds of 75mph+, extreme and unusual rainfall intensity) caused river to overflow and flood the caravan site; caravan floated 120 metres in flood water; damage caused by flood water immersion, not wind</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Holiday caravan</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Endorsement / Exclusion Challenge</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Declined — Full</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>Society of Lloyd's: policy expressly excluded 'all claims due to flood'; flood water caused the direct damage to the caravan; consumer himself described 'Storm Frank floated caravan 120 metres approx.' — confirming flood water as damaging agent, not wind; consumer was informed of flood exclusion approximately three years before the event and continued the policy</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>Consumer: storm conditions (which are covered) were the true cause of everything — storm caused flood which caused damage; storm is the proximate cause and should override the flood exclusion. Lloyd's: caravan was damaged by flood water not wind; consumer's own description confirms this; storm and flood are distinguishable events; policy clearly excluded all flood claims. FOS: weather records confirmed storm conditions (75mph gusts, extreme rainfall intensity) — qualifies as storm. But consumer's own statement ('floated caravan 120 metres') confirms flood water was the direct damaging cause; if caravan had been beyond reach of flood water, storm winds would not have caused the damage; proximate cause of loss = flood, not storm.</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>Not Upheld</t>
+        </is>
+      </c>
+      <c r="M56" s="3" t="inlineStr">
+        <is>
+          <t>Complaint not upheld; Lloyd's reasonably declined claim under the express 'all claims due to flood' exclusion; flood water was the proximate cause of loss; storm conditions were the antecedent cause not the direct cause of damage</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="P56" s="3" t="inlineStr">
+        <is>
+          <t>Explicit 'all claims due to flood' exclusion covers damage caused by flood water even when storm conditions caused the flood event; proximate cause rule — the immediate/direct cause of damage (flood water) determines which exclusion applies, not the antecedent cause (storm); consumer's own incident description is an important evidential admission about the actual mechanism of damage; consumer awareness of flood exclusion for approximately three years and continuation of policy = informed acceptance of exclusion terms; storm-triggered floods fall within a broad flood exclusion</t>
+        </is>
+      </c>
+      <c r="Q56" s="3" t="inlineStr">
+        <is>
+          <t>N/A — consumer's own description of the incident confirmed flood water as the direct cause; weather records verified storm conditions; damage extent confirmed to exceed sum insured</t>
+        </is>
+      </c>
+      <c r="R56" s="3" t="inlineStr">
+        <is>
+          <t>Weather records confirmed storm conditions (75mph+ gusts, extreme rainfall). Consumer himself reported 'Storm Frank floated caravan 120 metres approx.' — flood water was the direct damaging agent. FOS: storm caused river to burst banks (accepted), but it was the flood water that caused the loss. If caravan had been outside the flood's reach, storm winds alone would not have caused the damage. Proximate/immediate cause = flood. Policy excluded 'all claims due to flood' — broad exclusion covering storm-triggered flood events. Consumer knew about exclusion ~3 years before and continued the policy. Additional damage claim when caravan was moved irrelevant as total repair cost exceeded sum insured.</t>
+        </is>
+      </c>
+      <c r="S56" s="3" t="inlineStr">
+        <is>
+          <t>Where storm causes a flood which causes the damage, the immediate cause of damage (flood water) is the proximate cause — not the antecedent storm. A broad flood exclusion ('all claims due to flood') will encompass storm-triggered flood events and defeat arguments that storm cover should apply. Consumer's own description of the incident is a powerful admission: 'Storm Frank floated my caravan' confirms flood water was the damaging mechanism. Long-standing consumer awareness of an exclusion and continued policy renewal = acceptance of those exclusion terms. Additional damage claimed during recovery/removal is not separately recoverable if total repair cost exceeds sum insured.</t>
+        </is>
+      </c>
+      <c r="T56" s="3" t="inlineStr">
+        <is>
+          <t>IF storm_causes_flood_which_causes_damage AND policy_has_broad_flood_exclusion THEN flood_is_proximate_cause_and_exclusion_applies; storm_cover_does_not_override_express_flood_exclusion_where_flood_is_direct_damaging_mechanism; consumer_own_description_of_flood_water_as_damaging_agent_is_decisive_evidential_admission; consumer_awareness_of_flood_exclusion_for_multiple_years_and_policy_continuation_is_acceptance_of_exclusion_terms</t>
+        </is>
+      </c>
+      <c r="U56" s="2" t="inlineStr">
+        <is>
+          <t>DRN9771710.pdf</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>